<commit_message>
更新数据 + 修复SKU_INVENTORY shop|sku键映射
</commit_message>
<xml_diff>
--- a/2026WB年规进度 - 女装.xlsx
+++ b/2026WB年规进度 - 女装.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13380"/>
+    <workbookView windowWidth="29868" windowHeight="13380" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Z-NZTF1店" sheetId="9" r:id="rId1"/>
@@ -15,6 +15,7 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1386,6 +1387,1237 @@
     <sheetDataSet>
       <sheetData sheetId="0"/>
       <sheetData sheetId="1">
+        <row r="4">
+          <cell r="D4">
+            <v>9892</v>
+          </cell>
+          <cell r="E4">
+            <v>6207</v>
+          </cell>
+          <cell r="F4">
+            <v>6031</v>
+          </cell>
+          <cell r="G4">
+            <v>2483</v>
+          </cell>
+          <cell r="H4">
+            <v>0</v>
+          </cell>
+          <cell r="I4">
+            <v>0</v>
+          </cell>
+          <cell r="J4">
+            <v>0</v>
+          </cell>
+          <cell r="K4">
+            <v>0</v>
+          </cell>
+          <cell r="L4">
+            <v>0</v>
+          </cell>
+          <cell r="M4">
+            <v>0</v>
+          </cell>
+          <cell r="N4">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="C13">
+            <v>0</v>
+          </cell>
+          <cell r="D13">
+            <v>0</v>
+          </cell>
+          <cell r="E13">
+            <v>0</v>
+          </cell>
+          <cell r="F13">
+            <v>0</v>
+          </cell>
+          <cell r="G13">
+            <v>0</v>
+          </cell>
+          <cell r="H13">
+            <v>0</v>
+          </cell>
+          <cell r="I13">
+            <v>0</v>
+          </cell>
+          <cell r="J13">
+            <v>0</v>
+          </cell>
+          <cell r="K13">
+            <v>0</v>
+          </cell>
+          <cell r="L13">
+            <v>0</v>
+          </cell>
+          <cell r="M13">
+            <v>0</v>
+          </cell>
+          <cell r="N13">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="C14">
+            <v>0</v>
+          </cell>
+          <cell r="D14">
+            <v>0</v>
+          </cell>
+          <cell r="E14">
+            <v>0</v>
+          </cell>
+          <cell r="F14">
+            <v>0</v>
+          </cell>
+          <cell r="G14">
+            <v>0</v>
+          </cell>
+          <cell r="H14">
+            <v>0</v>
+          </cell>
+          <cell r="I14">
+            <v>0</v>
+          </cell>
+          <cell r="J14">
+            <v>0</v>
+          </cell>
+          <cell r="K14">
+            <v>0</v>
+          </cell>
+          <cell r="L14">
+            <v>0</v>
+          </cell>
+          <cell r="M14">
+            <v>0</v>
+          </cell>
+          <cell r="N14">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15">
+            <v>0</v>
+          </cell>
+          <cell r="D15">
+            <v>0</v>
+          </cell>
+          <cell r="E15">
+            <v>0</v>
+          </cell>
+          <cell r="F15">
+            <v>0</v>
+          </cell>
+          <cell r="G15">
+            <v>0</v>
+          </cell>
+          <cell r="H15">
+            <v>0</v>
+          </cell>
+          <cell r="I15">
+            <v>0</v>
+          </cell>
+          <cell r="J15">
+            <v>0</v>
+          </cell>
+          <cell r="K15">
+            <v>0</v>
+          </cell>
+          <cell r="L15">
+            <v>0</v>
+          </cell>
+          <cell r="M15">
+            <v>0</v>
+          </cell>
+          <cell r="N15">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="C16">
+            <v>0</v>
+          </cell>
+          <cell r="D16">
+            <v>0</v>
+          </cell>
+          <cell r="E16">
+            <v>0</v>
+          </cell>
+          <cell r="F16">
+            <v>0</v>
+          </cell>
+          <cell r="G16">
+            <v>0</v>
+          </cell>
+          <cell r="H16">
+            <v>0</v>
+          </cell>
+          <cell r="I16">
+            <v>0</v>
+          </cell>
+          <cell r="J16">
+            <v>0</v>
+          </cell>
+          <cell r="K16">
+            <v>0</v>
+          </cell>
+          <cell r="L16">
+            <v>0</v>
+          </cell>
+          <cell r="M16">
+            <v>0</v>
+          </cell>
+          <cell r="N16">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="C17">
+            <v>0</v>
+          </cell>
+          <cell r="D17">
+            <v>0</v>
+          </cell>
+          <cell r="E17">
+            <v>0</v>
+          </cell>
+          <cell r="F17">
+            <v>0</v>
+          </cell>
+          <cell r="G17">
+            <v>0</v>
+          </cell>
+          <cell r="H17">
+            <v>0</v>
+          </cell>
+          <cell r="I17">
+            <v>0</v>
+          </cell>
+          <cell r="J17">
+            <v>0</v>
+          </cell>
+          <cell r="K17">
+            <v>0</v>
+          </cell>
+          <cell r="L17">
+            <v>0</v>
+          </cell>
+          <cell r="M17">
+            <v>0</v>
+          </cell>
+          <cell r="N17">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="C18">
+            <v>0</v>
+          </cell>
+          <cell r="D18">
+            <v>0</v>
+          </cell>
+          <cell r="E18">
+            <v>0</v>
+          </cell>
+          <cell r="F18">
+            <v>0</v>
+          </cell>
+          <cell r="G18">
+            <v>0</v>
+          </cell>
+          <cell r="H18">
+            <v>0</v>
+          </cell>
+          <cell r="I18">
+            <v>0</v>
+          </cell>
+          <cell r="J18">
+            <v>0</v>
+          </cell>
+          <cell r="K18">
+            <v>0</v>
+          </cell>
+          <cell r="L18">
+            <v>0</v>
+          </cell>
+          <cell r="M18">
+            <v>0</v>
+          </cell>
+          <cell r="N18">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="C19">
+            <v>0</v>
+          </cell>
+          <cell r="D19">
+            <v>0</v>
+          </cell>
+          <cell r="E19">
+            <v>0</v>
+          </cell>
+          <cell r="F19">
+            <v>0</v>
+          </cell>
+          <cell r="G19">
+            <v>0</v>
+          </cell>
+          <cell r="H19">
+            <v>0</v>
+          </cell>
+          <cell r="I19">
+            <v>0</v>
+          </cell>
+          <cell r="J19">
+            <v>0</v>
+          </cell>
+          <cell r="K19">
+            <v>0</v>
+          </cell>
+          <cell r="L19">
+            <v>0</v>
+          </cell>
+          <cell r="M19">
+            <v>0</v>
+          </cell>
+          <cell r="N19">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="C20">
+            <v>0</v>
+          </cell>
+          <cell r="D20">
+            <v>0</v>
+          </cell>
+          <cell r="E20">
+            <v>0</v>
+          </cell>
+          <cell r="F20">
+            <v>0</v>
+          </cell>
+          <cell r="G20">
+            <v>0</v>
+          </cell>
+          <cell r="H20">
+            <v>0</v>
+          </cell>
+          <cell r="I20">
+            <v>0</v>
+          </cell>
+          <cell r="J20">
+            <v>0</v>
+          </cell>
+          <cell r="K20">
+            <v>0</v>
+          </cell>
+          <cell r="L20">
+            <v>0</v>
+          </cell>
+          <cell r="M20">
+            <v>0</v>
+          </cell>
+          <cell r="N20">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="C21">
+            <v>0</v>
+          </cell>
+          <cell r="D21">
+            <v>0</v>
+          </cell>
+          <cell r="E21">
+            <v>0</v>
+          </cell>
+          <cell r="F21">
+            <v>0</v>
+          </cell>
+          <cell r="G21">
+            <v>0</v>
+          </cell>
+          <cell r="H21">
+            <v>0</v>
+          </cell>
+          <cell r="I21">
+            <v>0</v>
+          </cell>
+          <cell r="J21">
+            <v>0</v>
+          </cell>
+          <cell r="K21">
+            <v>0</v>
+          </cell>
+          <cell r="L21">
+            <v>0</v>
+          </cell>
+          <cell r="M21">
+            <v>0</v>
+          </cell>
+          <cell r="N21">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="C22">
+            <v>0</v>
+          </cell>
+          <cell r="D22">
+            <v>0</v>
+          </cell>
+          <cell r="E22">
+            <v>0</v>
+          </cell>
+          <cell r="F22">
+            <v>0</v>
+          </cell>
+          <cell r="G22">
+            <v>0</v>
+          </cell>
+          <cell r="H22">
+            <v>0</v>
+          </cell>
+          <cell r="I22">
+            <v>0</v>
+          </cell>
+          <cell r="J22">
+            <v>0</v>
+          </cell>
+          <cell r="K22">
+            <v>0</v>
+          </cell>
+          <cell r="L22">
+            <v>0</v>
+          </cell>
+          <cell r="M22">
+            <v>0</v>
+          </cell>
+          <cell r="N22">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="C23">
+            <v>0</v>
+          </cell>
+          <cell r="D23">
+            <v>0</v>
+          </cell>
+          <cell r="E23">
+            <v>0</v>
+          </cell>
+          <cell r="F23">
+            <v>0</v>
+          </cell>
+          <cell r="G23">
+            <v>0</v>
+          </cell>
+          <cell r="H23">
+            <v>0</v>
+          </cell>
+          <cell r="I23">
+            <v>0</v>
+          </cell>
+          <cell r="J23">
+            <v>0</v>
+          </cell>
+          <cell r="K23">
+            <v>0</v>
+          </cell>
+          <cell r="L23">
+            <v>0</v>
+          </cell>
+          <cell r="M23">
+            <v>0</v>
+          </cell>
+          <cell r="N23">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="C24">
+            <v>0</v>
+          </cell>
+          <cell r="D24">
+            <v>0</v>
+          </cell>
+          <cell r="E24">
+            <v>0</v>
+          </cell>
+          <cell r="F24">
+            <v>0</v>
+          </cell>
+          <cell r="G24">
+            <v>0</v>
+          </cell>
+          <cell r="H24">
+            <v>0</v>
+          </cell>
+          <cell r="I24">
+            <v>0</v>
+          </cell>
+          <cell r="J24">
+            <v>0</v>
+          </cell>
+          <cell r="K24">
+            <v>0</v>
+          </cell>
+          <cell r="L24">
+            <v>0</v>
+          </cell>
+          <cell r="M24">
+            <v>0</v>
+          </cell>
+          <cell r="N24">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="C25">
+            <v>0</v>
+          </cell>
+          <cell r="D25">
+            <v>0</v>
+          </cell>
+          <cell r="E25">
+            <v>0</v>
+          </cell>
+          <cell r="F25">
+            <v>0</v>
+          </cell>
+          <cell r="G25">
+            <v>0</v>
+          </cell>
+          <cell r="H25">
+            <v>0</v>
+          </cell>
+          <cell r="I25">
+            <v>0</v>
+          </cell>
+          <cell r="J25">
+            <v>0</v>
+          </cell>
+          <cell r="K25">
+            <v>0</v>
+          </cell>
+          <cell r="L25">
+            <v>0</v>
+          </cell>
+          <cell r="M25">
+            <v>0</v>
+          </cell>
+          <cell r="N25">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="C26">
+            <v>0</v>
+          </cell>
+          <cell r="D26">
+            <v>0</v>
+          </cell>
+          <cell r="E26">
+            <v>0</v>
+          </cell>
+          <cell r="F26">
+            <v>0</v>
+          </cell>
+          <cell r="G26">
+            <v>0</v>
+          </cell>
+          <cell r="H26">
+            <v>0</v>
+          </cell>
+          <cell r="I26">
+            <v>0</v>
+          </cell>
+          <cell r="J26">
+            <v>0</v>
+          </cell>
+          <cell r="K26">
+            <v>0</v>
+          </cell>
+          <cell r="L26">
+            <v>0</v>
+          </cell>
+          <cell r="M26">
+            <v>0</v>
+          </cell>
+          <cell r="N26">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="C27">
+            <v>0</v>
+          </cell>
+          <cell r="D27">
+            <v>0</v>
+          </cell>
+          <cell r="E27">
+            <v>0</v>
+          </cell>
+          <cell r="F27">
+            <v>0</v>
+          </cell>
+          <cell r="G27">
+            <v>0</v>
+          </cell>
+          <cell r="H27">
+            <v>0</v>
+          </cell>
+          <cell r="I27">
+            <v>0</v>
+          </cell>
+          <cell r="J27">
+            <v>0</v>
+          </cell>
+          <cell r="K27">
+            <v>0</v>
+          </cell>
+          <cell r="L27">
+            <v>0</v>
+          </cell>
+          <cell r="M27">
+            <v>0</v>
+          </cell>
+          <cell r="N27">
+            <v>0</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3">
+        <row r="29">
+          <cell r="C29">
+            <v>3997.42101869763</v>
+          </cell>
+          <cell r="D29">
+            <v>7736.94390715666</v>
+          </cell>
+          <cell r="E29">
+            <v>7994.84203739522</v>
+          </cell>
+          <cell r="F29">
+            <v>7736.94390715666</v>
+          </cell>
+          <cell r="G29">
+            <v>7994.84203739522</v>
+          </cell>
+          <cell r="H29">
+            <v>13990.9735654417</v>
+          </cell>
+          <cell r="I29">
+            <v>13539.6518375242</v>
+          </cell>
+          <cell r="J29">
+            <v>11992.2630560929</v>
+          </cell>
+          <cell r="K29">
+            <v>11605.415860735</v>
+          </cell>
+          <cell r="L29">
+            <v>11992.2630560929</v>
+          </cell>
+          <cell r="M29">
+            <v>5996.13152804641</v>
+          </cell>
+        </row>
+        <row r="55">
+          <cell r="B55">
+            <v>0</v>
+          </cell>
+          <cell r="C55">
+            <v>0</v>
+          </cell>
+          <cell r="D55">
+            <v>0</v>
+          </cell>
+          <cell r="E55">
+            <v>0</v>
+          </cell>
+          <cell r="F55">
+            <v>0</v>
+          </cell>
+          <cell r="G55">
+            <v>0</v>
+          </cell>
+          <cell r="H55">
+            <v>0</v>
+          </cell>
+          <cell r="I55">
+            <v>26785714.2857143</v>
+          </cell>
+          <cell r="J55">
+            <v>35714285.7142857</v>
+          </cell>
+          <cell r="K55">
+            <v>44642857.1428571</v>
+          </cell>
+          <cell r="L55">
+            <v>44642857.1428571</v>
+          </cell>
+          <cell r="M55">
+            <v>26785714.2857143</v>
+          </cell>
+        </row>
+        <row r="57">
+          <cell r="B57">
+            <v>0</v>
+          </cell>
+          <cell r="C57">
+            <v>0</v>
+          </cell>
+          <cell r="D57">
+            <v>0</v>
+          </cell>
+          <cell r="E57">
+            <v>0</v>
+          </cell>
+          <cell r="F57">
+            <v>0</v>
+          </cell>
+          <cell r="G57">
+            <v>0</v>
+          </cell>
+          <cell r="H57">
+            <v>0</v>
+          </cell>
+          <cell r="I57">
+            <v>450000</v>
+          </cell>
+          <cell r="J57">
+            <v>600000</v>
+          </cell>
+          <cell r="K57">
+            <v>750000</v>
+          </cell>
+          <cell r="L57">
+            <v>750000</v>
+          </cell>
+          <cell r="M57">
+            <v>450000</v>
+          </cell>
+        </row>
+        <row r="59">
+          <cell r="B59">
+            <v>0</v>
+          </cell>
+          <cell r="C59">
+            <v>0</v>
+          </cell>
+          <cell r="D59">
+            <v>0</v>
+          </cell>
+          <cell r="E59">
+            <v>0</v>
+          </cell>
+          <cell r="F59">
+            <v>0</v>
+          </cell>
+          <cell r="G59">
+            <v>0</v>
+          </cell>
+          <cell r="H59">
+            <v>0</v>
+          </cell>
+          <cell r="I59">
+            <v>45000</v>
+          </cell>
+          <cell r="J59">
+            <v>60000</v>
+          </cell>
+          <cell r="K59">
+            <v>75000</v>
+          </cell>
+          <cell r="L59">
+            <v>75000</v>
+          </cell>
+          <cell r="M59">
+            <v>45000</v>
+          </cell>
+        </row>
+        <row r="63">
+          <cell r="B63">
+            <v>0</v>
+          </cell>
+          <cell r="C63">
+            <v>0</v>
+          </cell>
+          <cell r="D63">
+            <v>0</v>
+          </cell>
+          <cell r="E63">
+            <v>0</v>
+          </cell>
+          <cell r="F63">
+            <v>0</v>
+          </cell>
+          <cell r="G63">
+            <v>0</v>
+          </cell>
+          <cell r="H63">
+            <v>0</v>
+          </cell>
+          <cell r="I63">
+            <v>5699.08814589666</v>
+          </cell>
+          <cell r="J63">
+            <v>7598.78419452888</v>
+          </cell>
+          <cell r="K63">
+            <v>9498.4802431611</v>
+          </cell>
+          <cell r="L63">
+            <v>9498.4802431611</v>
+          </cell>
+          <cell r="M63">
+            <v>5699.08814589666</v>
+          </cell>
+        </row>
+        <row r="65">
+          <cell r="B65">
+            <v>0</v>
+          </cell>
+          <cell r="C65">
+            <v>0</v>
+          </cell>
+          <cell r="D65">
+            <v>0</v>
+          </cell>
+          <cell r="E65">
+            <v>0</v>
+          </cell>
+          <cell r="F65">
+            <v>0</v>
+          </cell>
+          <cell r="G65">
+            <v>0</v>
+          </cell>
+          <cell r="H65">
+            <v>0</v>
+          </cell>
+          <cell r="I65">
+            <v>1196.8085106383</v>
+          </cell>
+          <cell r="J65">
+            <v>1595.74468085106</v>
+          </cell>
+          <cell r="K65">
+            <v>1994.68085106383</v>
+          </cell>
+          <cell r="L65">
+            <v>1994.68085106383</v>
+          </cell>
+          <cell r="M65">
+            <v>1196.8085106383</v>
+          </cell>
+        </row>
+        <row r="72">
+          <cell r="B72">
+            <v>0</v>
+          </cell>
+          <cell r="C72">
+            <v>0</v>
+          </cell>
+          <cell r="D72">
+            <v>0</v>
+          </cell>
+          <cell r="E72">
+            <v>0</v>
+          </cell>
+          <cell r="F72">
+            <v>0</v>
+          </cell>
+          <cell r="G72">
+            <v>0</v>
+          </cell>
+          <cell r="H72">
+            <v>21428571.4285714</v>
+          </cell>
+          <cell r="I72">
+            <v>64285714.2857143</v>
+          </cell>
+          <cell r="J72">
+            <v>89285714.2857143</v>
+          </cell>
+          <cell r="K72">
+            <v>89285714.2857143</v>
+          </cell>
+          <cell r="L72">
+            <v>71428571.4285714</v>
+          </cell>
+          <cell r="M72">
+            <v>21428571.4285714</v>
+          </cell>
+        </row>
+        <row r="74">
+          <cell r="B74">
+            <v>0</v>
+          </cell>
+          <cell r="C74">
+            <v>0</v>
+          </cell>
+          <cell r="D74">
+            <v>0</v>
+          </cell>
+          <cell r="E74">
+            <v>0</v>
+          </cell>
+          <cell r="F74">
+            <v>0</v>
+          </cell>
+          <cell r="G74">
+            <v>0</v>
+          </cell>
+          <cell r="H74">
+            <v>360000</v>
+          </cell>
+          <cell r="I74">
+            <v>1080000</v>
+          </cell>
+          <cell r="J74">
+            <v>1500000</v>
+          </cell>
+          <cell r="K74">
+            <v>1500000</v>
+          </cell>
+          <cell r="L74">
+            <v>1200000</v>
+          </cell>
+          <cell r="M74">
+            <v>360000</v>
+          </cell>
+        </row>
+        <row r="76">
+          <cell r="B76">
+            <v>0</v>
+          </cell>
+          <cell r="C76">
+            <v>0</v>
+          </cell>
+          <cell r="D76">
+            <v>0</v>
+          </cell>
+          <cell r="E76">
+            <v>0</v>
+          </cell>
+          <cell r="F76">
+            <v>0</v>
+          </cell>
+          <cell r="G76">
+            <v>0</v>
+          </cell>
+          <cell r="H76">
+            <v>55080</v>
+          </cell>
+          <cell r="I76">
+            <v>165240</v>
+          </cell>
+          <cell r="J76">
+            <v>229500</v>
+          </cell>
+          <cell r="K76">
+            <v>229500</v>
+          </cell>
+          <cell r="L76">
+            <v>183600</v>
+          </cell>
+          <cell r="M76">
+            <v>55080</v>
+          </cell>
+        </row>
+        <row r="80">
+          <cell r="B80">
+            <v>0</v>
+          </cell>
+          <cell r="C80">
+            <v>0</v>
+          </cell>
+          <cell r="D80">
+            <v>0</v>
+          </cell>
+          <cell r="E80">
+            <v>0</v>
+          </cell>
+          <cell r="F80">
+            <v>0</v>
+          </cell>
+          <cell r="G80">
+            <v>0</v>
+          </cell>
+          <cell r="H80">
+            <v>4559.27051671733</v>
+          </cell>
+          <cell r="I80">
+            <v>13677.811550152</v>
+          </cell>
+          <cell r="J80">
+            <v>18996.9604863222</v>
+          </cell>
+          <cell r="K80">
+            <v>18996.9604863222</v>
+          </cell>
+          <cell r="L80">
+            <v>15197.5683890578</v>
+          </cell>
+          <cell r="M80">
+            <v>4559.27051671733</v>
+          </cell>
+        </row>
+        <row r="82">
+          <cell r="B82">
+            <v>0</v>
+          </cell>
+          <cell r="C82">
+            <v>0</v>
+          </cell>
+          <cell r="D82">
+            <v>0</v>
+          </cell>
+          <cell r="E82">
+            <v>0</v>
+          </cell>
+          <cell r="F82">
+            <v>0</v>
+          </cell>
+          <cell r="G82">
+            <v>0</v>
+          </cell>
+          <cell r="H82">
+            <v>957.446808510638</v>
+          </cell>
+          <cell r="I82">
+            <v>2872.34042553191</v>
+          </cell>
+          <cell r="J82">
+            <v>3989.36170212766</v>
+          </cell>
+          <cell r="K82">
+            <v>3989.36170212766</v>
+          </cell>
+          <cell r="L82">
+            <v>3191.48936170213</v>
+          </cell>
+          <cell r="M82">
+            <v>957.446808510638</v>
+          </cell>
+        </row>
+        <row r="89">
+          <cell r="B89">
+            <v>0</v>
+          </cell>
+          <cell r="C89">
+            <v>0</v>
+          </cell>
+          <cell r="D89">
+            <v>0</v>
+          </cell>
+          <cell r="E89">
+            <v>0</v>
+          </cell>
+          <cell r="F89">
+            <v>0</v>
+          </cell>
+          <cell r="G89">
+            <v>0</v>
+          </cell>
+          <cell r="H89">
+            <v>21428571.4285714</v>
+          </cell>
+          <cell r="I89">
+            <v>35714285.7142857</v>
+          </cell>
+          <cell r="J89">
+            <v>32142857.1428571</v>
+          </cell>
+          <cell r="K89">
+            <v>32142857.1428571</v>
+          </cell>
+          <cell r="L89">
+            <v>32142857.1428571</v>
+          </cell>
+          <cell r="M89">
+            <v>25000000</v>
+          </cell>
+        </row>
+        <row r="91">
+          <cell r="B91">
+            <v>0</v>
+          </cell>
+          <cell r="C91">
+            <v>0</v>
+          </cell>
+          <cell r="D91">
+            <v>0</v>
+          </cell>
+          <cell r="E91">
+            <v>0</v>
+          </cell>
+          <cell r="F91">
+            <v>0</v>
+          </cell>
+          <cell r="G91">
+            <v>0</v>
+          </cell>
+          <cell r="H91">
+            <v>360000</v>
+          </cell>
+          <cell r="I91">
+            <v>600000</v>
+          </cell>
+          <cell r="J91">
+            <v>540000</v>
+          </cell>
+          <cell r="K91">
+            <v>540000</v>
+          </cell>
+          <cell r="L91">
+            <v>540000</v>
+          </cell>
+          <cell r="M91">
+            <v>420000</v>
+          </cell>
+        </row>
+        <row r="93">
+          <cell r="B93">
+            <v>0</v>
+          </cell>
+          <cell r="C93">
+            <v>0</v>
+          </cell>
+          <cell r="D93">
+            <v>0</v>
+          </cell>
+          <cell r="E93">
+            <v>0</v>
+          </cell>
+          <cell r="F93">
+            <v>0</v>
+          </cell>
+          <cell r="G93">
+            <v>0</v>
+          </cell>
+          <cell r="H93">
+            <v>36000</v>
+          </cell>
+          <cell r="I93">
+            <v>60000</v>
+          </cell>
+          <cell r="J93">
+            <v>54000</v>
+          </cell>
+          <cell r="K93">
+            <v>54000</v>
+          </cell>
+          <cell r="L93">
+            <v>54000</v>
+          </cell>
+          <cell r="M93">
+            <v>42000</v>
+          </cell>
+        </row>
+        <row r="97">
+          <cell r="B97">
+            <v>0</v>
+          </cell>
+          <cell r="C97">
+            <v>0</v>
+          </cell>
+          <cell r="D97">
+            <v>0</v>
+          </cell>
+          <cell r="E97">
+            <v>0</v>
+          </cell>
+          <cell r="F97">
+            <v>0</v>
+          </cell>
+          <cell r="G97">
+            <v>0</v>
+          </cell>
+          <cell r="H97">
+            <v>4559.27051671733</v>
+          </cell>
+          <cell r="I97">
+            <v>7598.78419452888</v>
+          </cell>
+          <cell r="J97">
+            <v>6838.90577507599</v>
+          </cell>
+          <cell r="K97">
+            <v>6838.90577507599</v>
+          </cell>
+          <cell r="L97">
+            <v>6838.90577507599</v>
+          </cell>
+          <cell r="M97">
+            <v>5319.14893617021</v>
+          </cell>
+        </row>
+        <row r="99">
+          <cell r="B99">
+            <v>0</v>
+          </cell>
+          <cell r="C99">
+            <v>0</v>
+          </cell>
+          <cell r="D99">
+            <v>0</v>
+          </cell>
+          <cell r="E99">
+            <v>0</v>
+          </cell>
+          <cell r="F99">
+            <v>0</v>
+          </cell>
+          <cell r="G99">
+            <v>0</v>
+          </cell>
+          <cell r="H99">
+            <v>957.446808510638</v>
+          </cell>
+          <cell r="I99">
+            <v>1595.74468085106</v>
+          </cell>
+          <cell r="J99">
+            <v>1436.17021276596</v>
+          </cell>
+          <cell r="K99">
+            <v>1436.17021276596</v>
+          </cell>
+          <cell r="L99">
+            <v>1436.17021276596</v>
+          </cell>
+          <cell r="M99">
+            <v>1117.02127659574</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="年度数据汇总进度"/>
+      <sheetName val="月度数据汇总--女装"/>
+      <sheetName val="周度数据填报"/>
+      <sheetName val="目标拆解"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
         <row r="3">
           <cell r="C3">
             <v>-6740.65</v>
@@ -1400,10 +2632,10 @@
             <v>27181.29</v>
           </cell>
           <cell r="G3">
-            <v>-13699.74</v>
+            <v>-76428.1812484271</v>
           </cell>
           <cell r="H3">
-            <v>0</v>
+            <v>6257.5640211776</v>
           </cell>
           <cell r="I3">
             <v>0</v>
@@ -1428,39 +2660,6 @@
           <cell r="C4">
             <v>2362</v>
           </cell>
-          <cell r="D4">
-            <v>9892</v>
-          </cell>
-          <cell r="E4">
-            <v>6207</v>
-          </cell>
-          <cell r="F4">
-            <v>6031</v>
-          </cell>
-          <cell r="G4">
-            <v>2483</v>
-          </cell>
-          <cell r="H4">
-            <v>0</v>
-          </cell>
-          <cell r="I4">
-            <v>0</v>
-          </cell>
-          <cell r="J4">
-            <v>0</v>
-          </cell>
-          <cell r="K4">
-            <v>0</v>
-          </cell>
-          <cell r="L4">
-            <v>0</v>
-          </cell>
-          <cell r="M4">
-            <v>0</v>
-          </cell>
-          <cell r="N4">
-            <v>0</v>
-          </cell>
         </row>
         <row r="5">
           <cell r="C5">
@@ -1476,10 +2675,10 @@
             <v>1147</v>
           </cell>
           <cell r="G5">
-            <v>510</v>
+            <v>991</v>
           </cell>
           <cell r="H5">
-            <v>0</v>
+            <v>216</v>
           </cell>
           <cell r="I5">
             <v>0</v>
@@ -1514,10 +2713,10 @@
             <v>32616432</v>
           </cell>
           <cell r="G6">
-            <v>11981910</v>
+            <v>22407232</v>
           </cell>
           <cell r="H6">
-            <v>0</v>
+            <v>4613093</v>
           </cell>
           <cell r="I6">
             <v>0</v>
@@ -1552,10 +2751,10 @@
             <v>550489.45</v>
           </cell>
           <cell r="G7">
-            <v>238074.01</v>
+            <v>460996.035</v>
           </cell>
           <cell r="H7">
-            <v>0</v>
+            <v>94048.8148</v>
           </cell>
           <cell r="I7">
             <v>0</v>
@@ -1590,10 +2789,10 @@
             <v>154982.1</v>
           </cell>
           <cell r="G8">
-            <v>33716.99</v>
+            <v>58803.505650204</v>
           </cell>
           <cell r="H8">
-            <v>0</v>
+            <v>11848.3851122148</v>
           </cell>
           <cell r="I8">
             <v>0</v>
@@ -1628,10 +2827,10 @@
             <v>11196</v>
           </cell>
           <cell r="G9">
-            <v>4045</v>
+            <v>7971</v>
           </cell>
           <cell r="H9">
-            <v>0</v>
+            <v>1339</v>
           </cell>
           <cell r="I9">
             <v>0</v>
@@ -1666,10 +2865,10 @@
             <v>2441</v>
           </cell>
           <cell r="G10">
-            <v>887</v>
+            <v>1758</v>
           </cell>
           <cell r="H10">
-            <v>0</v>
+            <v>446</v>
           </cell>
           <cell r="I10">
             <v>0</v>
@@ -1704,10 +2903,10 @@
             <v>56092797</v>
           </cell>
           <cell r="G11">
-            <v>18377548</v>
+            <v>36922189</v>
           </cell>
           <cell r="H11">
-            <v>0</v>
+            <v>8733473</v>
           </cell>
           <cell r="I11">
             <v>0</v>
@@ -1742,10 +2941,10 @@
             <v>1069518.42</v>
           </cell>
           <cell r="G12">
-            <v>401111.57</v>
+            <v>797308.5406</v>
           </cell>
           <cell r="H12">
-            <v>0</v>
+            <v>192321.5225</v>
           </cell>
           <cell r="I12">
             <v>0</v>
@@ -1763,576 +2962,6 @@
             <v>0</v>
           </cell>
           <cell r="N12">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="C13">
-            <v>0</v>
-          </cell>
-          <cell r="D13">
-            <v>0</v>
-          </cell>
-          <cell r="E13">
-            <v>0</v>
-          </cell>
-          <cell r="F13">
-            <v>0</v>
-          </cell>
-          <cell r="G13">
-            <v>0</v>
-          </cell>
-          <cell r="H13">
-            <v>0</v>
-          </cell>
-          <cell r="I13">
-            <v>0</v>
-          </cell>
-          <cell r="J13">
-            <v>0</v>
-          </cell>
-          <cell r="K13">
-            <v>0</v>
-          </cell>
-          <cell r="L13">
-            <v>0</v>
-          </cell>
-          <cell r="M13">
-            <v>0</v>
-          </cell>
-          <cell r="N13">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="C14">
-            <v>0</v>
-          </cell>
-          <cell r="D14">
-            <v>0</v>
-          </cell>
-          <cell r="E14">
-            <v>0</v>
-          </cell>
-          <cell r="F14">
-            <v>0</v>
-          </cell>
-          <cell r="G14">
-            <v>0</v>
-          </cell>
-          <cell r="H14">
-            <v>0</v>
-          </cell>
-          <cell r="I14">
-            <v>0</v>
-          </cell>
-          <cell r="J14">
-            <v>0</v>
-          </cell>
-          <cell r="K14">
-            <v>0</v>
-          </cell>
-          <cell r="L14">
-            <v>0</v>
-          </cell>
-          <cell r="M14">
-            <v>0</v>
-          </cell>
-          <cell r="N14">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="C15">
-            <v>0</v>
-          </cell>
-          <cell r="D15">
-            <v>0</v>
-          </cell>
-          <cell r="E15">
-            <v>0</v>
-          </cell>
-          <cell r="F15">
-            <v>0</v>
-          </cell>
-          <cell r="G15">
-            <v>0</v>
-          </cell>
-          <cell r="H15">
-            <v>0</v>
-          </cell>
-          <cell r="I15">
-            <v>0</v>
-          </cell>
-          <cell r="J15">
-            <v>0</v>
-          </cell>
-          <cell r="K15">
-            <v>0</v>
-          </cell>
-          <cell r="L15">
-            <v>0</v>
-          </cell>
-          <cell r="M15">
-            <v>0</v>
-          </cell>
-          <cell r="N15">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="C16">
-            <v>0</v>
-          </cell>
-          <cell r="D16">
-            <v>0</v>
-          </cell>
-          <cell r="E16">
-            <v>0</v>
-          </cell>
-          <cell r="F16">
-            <v>0</v>
-          </cell>
-          <cell r="G16">
-            <v>0</v>
-          </cell>
-          <cell r="H16">
-            <v>0</v>
-          </cell>
-          <cell r="I16">
-            <v>0</v>
-          </cell>
-          <cell r="J16">
-            <v>0</v>
-          </cell>
-          <cell r="K16">
-            <v>0</v>
-          </cell>
-          <cell r="L16">
-            <v>0</v>
-          </cell>
-          <cell r="M16">
-            <v>0</v>
-          </cell>
-          <cell r="N16">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="C17">
-            <v>0</v>
-          </cell>
-          <cell r="D17">
-            <v>0</v>
-          </cell>
-          <cell r="E17">
-            <v>0</v>
-          </cell>
-          <cell r="F17">
-            <v>0</v>
-          </cell>
-          <cell r="G17">
-            <v>0</v>
-          </cell>
-          <cell r="H17">
-            <v>0</v>
-          </cell>
-          <cell r="I17">
-            <v>0</v>
-          </cell>
-          <cell r="J17">
-            <v>0</v>
-          </cell>
-          <cell r="K17">
-            <v>0</v>
-          </cell>
-          <cell r="L17">
-            <v>0</v>
-          </cell>
-          <cell r="M17">
-            <v>0</v>
-          </cell>
-          <cell r="N17">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="C18">
-            <v>0</v>
-          </cell>
-          <cell r="D18">
-            <v>0</v>
-          </cell>
-          <cell r="E18">
-            <v>0</v>
-          </cell>
-          <cell r="F18">
-            <v>0</v>
-          </cell>
-          <cell r="G18">
-            <v>0</v>
-          </cell>
-          <cell r="H18">
-            <v>0</v>
-          </cell>
-          <cell r="I18">
-            <v>0</v>
-          </cell>
-          <cell r="J18">
-            <v>0</v>
-          </cell>
-          <cell r="K18">
-            <v>0</v>
-          </cell>
-          <cell r="L18">
-            <v>0</v>
-          </cell>
-          <cell r="M18">
-            <v>0</v>
-          </cell>
-          <cell r="N18">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="C19">
-            <v>0</v>
-          </cell>
-          <cell r="D19">
-            <v>0</v>
-          </cell>
-          <cell r="E19">
-            <v>0</v>
-          </cell>
-          <cell r="F19">
-            <v>0</v>
-          </cell>
-          <cell r="G19">
-            <v>0</v>
-          </cell>
-          <cell r="H19">
-            <v>0</v>
-          </cell>
-          <cell r="I19">
-            <v>0</v>
-          </cell>
-          <cell r="J19">
-            <v>0</v>
-          </cell>
-          <cell r="K19">
-            <v>0</v>
-          </cell>
-          <cell r="L19">
-            <v>0</v>
-          </cell>
-          <cell r="M19">
-            <v>0</v>
-          </cell>
-          <cell r="N19">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="C20">
-            <v>0</v>
-          </cell>
-          <cell r="D20">
-            <v>0</v>
-          </cell>
-          <cell r="E20">
-            <v>0</v>
-          </cell>
-          <cell r="F20">
-            <v>0</v>
-          </cell>
-          <cell r="G20">
-            <v>0</v>
-          </cell>
-          <cell r="H20">
-            <v>0</v>
-          </cell>
-          <cell r="I20">
-            <v>0</v>
-          </cell>
-          <cell r="J20">
-            <v>0</v>
-          </cell>
-          <cell r="K20">
-            <v>0</v>
-          </cell>
-          <cell r="L20">
-            <v>0</v>
-          </cell>
-          <cell r="M20">
-            <v>0</v>
-          </cell>
-          <cell r="N20">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="C21">
-            <v>0</v>
-          </cell>
-          <cell r="D21">
-            <v>0</v>
-          </cell>
-          <cell r="E21">
-            <v>0</v>
-          </cell>
-          <cell r="F21">
-            <v>0</v>
-          </cell>
-          <cell r="G21">
-            <v>0</v>
-          </cell>
-          <cell r="H21">
-            <v>0</v>
-          </cell>
-          <cell r="I21">
-            <v>0</v>
-          </cell>
-          <cell r="J21">
-            <v>0</v>
-          </cell>
-          <cell r="K21">
-            <v>0</v>
-          </cell>
-          <cell r="L21">
-            <v>0</v>
-          </cell>
-          <cell r="M21">
-            <v>0</v>
-          </cell>
-          <cell r="N21">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="C22">
-            <v>0</v>
-          </cell>
-          <cell r="D22">
-            <v>0</v>
-          </cell>
-          <cell r="E22">
-            <v>0</v>
-          </cell>
-          <cell r="F22">
-            <v>0</v>
-          </cell>
-          <cell r="G22">
-            <v>0</v>
-          </cell>
-          <cell r="H22">
-            <v>0</v>
-          </cell>
-          <cell r="I22">
-            <v>0</v>
-          </cell>
-          <cell r="J22">
-            <v>0</v>
-          </cell>
-          <cell r="K22">
-            <v>0</v>
-          </cell>
-          <cell r="L22">
-            <v>0</v>
-          </cell>
-          <cell r="M22">
-            <v>0</v>
-          </cell>
-          <cell r="N22">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="C23">
-            <v>0</v>
-          </cell>
-          <cell r="D23">
-            <v>0</v>
-          </cell>
-          <cell r="E23">
-            <v>0</v>
-          </cell>
-          <cell r="F23">
-            <v>0</v>
-          </cell>
-          <cell r="G23">
-            <v>0</v>
-          </cell>
-          <cell r="H23">
-            <v>0</v>
-          </cell>
-          <cell r="I23">
-            <v>0</v>
-          </cell>
-          <cell r="J23">
-            <v>0</v>
-          </cell>
-          <cell r="K23">
-            <v>0</v>
-          </cell>
-          <cell r="L23">
-            <v>0</v>
-          </cell>
-          <cell r="M23">
-            <v>0</v>
-          </cell>
-          <cell r="N23">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="C24">
-            <v>0</v>
-          </cell>
-          <cell r="D24">
-            <v>0</v>
-          </cell>
-          <cell r="E24">
-            <v>0</v>
-          </cell>
-          <cell r="F24">
-            <v>0</v>
-          </cell>
-          <cell r="G24">
-            <v>0</v>
-          </cell>
-          <cell r="H24">
-            <v>0</v>
-          </cell>
-          <cell r="I24">
-            <v>0</v>
-          </cell>
-          <cell r="J24">
-            <v>0</v>
-          </cell>
-          <cell r="K24">
-            <v>0</v>
-          </cell>
-          <cell r="L24">
-            <v>0</v>
-          </cell>
-          <cell r="M24">
-            <v>0</v>
-          </cell>
-          <cell r="N24">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="C25">
-            <v>0</v>
-          </cell>
-          <cell r="D25">
-            <v>0</v>
-          </cell>
-          <cell r="E25">
-            <v>0</v>
-          </cell>
-          <cell r="F25">
-            <v>0</v>
-          </cell>
-          <cell r="G25">
-            <v>0</v>
-          </cell>
-          <cell r="H25">
-            <v>0</v>
-          </cell>
-          <cell r="I25">
-            <v>0</v>
-          </cell>
-          <cell r="J25">
-            <v>0</v>
-          </cell>
-          <cell r="K25">
-            <v>0</v>
-          </cell>
-          <cell r="L25">
-            <v>0</v>
-          </cell>
-          <cell r="M25">
-            <v>0</v>
-          </cell>
-          <cell r="N25">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="C26">
-            <v>0</v>
-          </cell>
-          <cell r="D26">
-            <v>0</v>
-          </cell>
-          <cell r="E26">
-            <v>0</v>
-          </cell>
-          <cell r="F26">
-            <v>0</v>
-          </cell>
-          <cell r="G26">
-            <v>0</v>
-          </cell>
-          <cell r="H26">
-            <v>0</v>
-          </cell>
-          <cell r="I26">
-            <v>0</v>
-          </cell>
-          <cell r="J26">
-            <v>0</v>
-          </cell>
-          <cell r="K26">
-            <v>0</v>
-          </cell>
-          <cell r="L26">
-            <v>0</v>
-          </cell>
-          <cell r="M26">
-            <v>0</v>
-          </cell>
-          <cell r="N26">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="C27">
-            <v>0</v>
-          </cell>
-          <cell r="D27">
-            <v>0</v>
-          </cell>
-          <cell r="E27">
-            <v>0</v>
-          </cell>
-          <cell r="F27">
-            <v>0</v>
-          </cell>
-          <cell r="G27">
-            <v>0</v>
-          </cell>
-          <cell r="H27">
-            <v>0</v>
-          </cell>
-          <cell r="I27">
-            <v>0</v>
-          </cell>
-          <cell r="J27">
-            <v>0</v>
-          </cell>
-          <cell r="K27">
-            <v>0</v>
-          </cell>
-          <cell r="L27">
-            <v>0</v>
-          </cell>
-          <cell r="M27">
-            <v>0</v>
-          </cell>
-          <cell r="N27">
             <v>0</v>
           </cell>
         </row>
@@ -2457,39 +3086,6 @@
           <cell r="B29">
             <v>1805.28691166989</v>
           </cell>
-          <cell r="C29">
-            <v>3997.42101869763</v>
-          </cell>
-          <cell r="D29">
-            <v>7736.94390715666</v>
-          </cell>
-          <cell r="E29">
-            <v>7994.84203739522</v>
-          </cell>
-          <cell r="F29">
-            <v>7736.94390715666</v>
-          </cell>
-          <cell r="G29">
-            <v>7994.84203739522</v>
-          </cell>
-          <cell r="H29">
-            <v>13990.9735654417</v>
-          </cell>
-          <cell r="I29">
-            <v>13539.6518375242</v>
-          </cell>
-          <cell r="J29">
-            <v>11992.2630560929</v>
-          </cell>
-          <cell r="K29">
-            <v>11605.415860735</v>
-          </cell>
-          <cell r="L29">
-            <v>11992.2630560929</v>
-          </cell>
-          <cell r="M29">
-            <v>5996.13152804641</v>
-          </cell>
         </row>
         <row r="31">
           <cell r="B31">
@@ -2679,576 +3275,6 @@
           </cell>
           <cell r="M46">
             <v>6813.78582732546</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="B55">
-            <v>0</v>
-          </cell>
-          <cell r="C55">
-            <v>0</v>
-          </cell>
-          <cell r="D55">
-            <v>0</v>
-          </cell>
-          <cell r="E55">
-            <v>0</v>
-          </cell>
-          <cell r="F55">
-            <v>0</v>
-          </cell>
-          <cell r="G55">
-            <v>0</v>
-          </cell>
-          <cell r="H55">
-            <v>0</v>
-          </cell>
-          <cell r="I55">
-            <v>26785714.2857143</v>
-          </cell>
-          <cell r="J55">
-            <v>35714285.7142857</v>
-          </cell>
-          <cell r="K55">
-            <v>44642857.1428571</v>
-          </cell>
-          <cell r="L55">
-            <v>44642857.1428571</v>
-          </cell>
-          <cell r="M55">
-            <v>26785714.2857143</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="B57">
-            <v>0</v>
-          </cell>
-          <cell r="C57">
-            <v>0</v>
-          </cell>
-          <cell r="D57">
-            <v>0</v>
-          </cell>
-          <cell r="E57">
-            <v>0</v>
-          </cell>
-          <cell r="F57">
-            <v>0</v>
-          </cell>
-          <cell r="G57">
-            <v>0</v>
-          </cell>
-          <cell r="H57">
-            <v>0</v>
-          </cell>
-          <cell r="I57">
-            <v>450000</v>
-          </cell>
-          <cell r="J57">
-            <v>600000</v>
-          </cell>
-          <cell r="K57">
-            <v>750000</v>
-          </cell>
-          <cell r="L57">
-            <v>750000</v>
-          </cell>
-          <cell r="M57">
-            <v>450000</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="B59">
-            <v>0</v>
-          </cell>
-          <cell r="C59">
-            <v>0</v>
-          </cell>
-          <cell r="D59">
-            <v>0</v>
-          </cell>
-          <cell r="E59">
-            <v>0</v>
-          </cell>
-          <cell r="F59">
-            <v>0</v>
-          </cell>
-          <cell r="G59">
-            <v>0</v>
-          </cell>
-          <cell r="H59">
-            <v>0</v>
-          </cell>
-          <cell r="I59">
-            <v>45000</v>
-          </cell>
-          <cell r="J59">
-            <v>60000</v>
-          </cell>
-          <cell r="K59">
-            <v>75000</v>
-          </cell>
-          <cell r="L59">
-            <v>75000</v>
-          </cell>
-          <cell r="M59">
-            <v>45000</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="B63">
-            <v>0</v>
-          </cell>
-          <cell r="C63">
-            <v>0</v>
-          </cell>
-          <cell r="D63">
-            <v>0</v>
-          </cell>
-          <cell r="E63">
-            <v>0</v>
-          </cell>
-          <cell r="F63">
-            <v>0</v>
-          </cell>
-          <cell r="G63">
-            <v>0</v>
-          </cell>
-          <cell r="H63">
-            <v>0</v>
-          </cell>
-          <cell r="I63">
-            <v>5699.08814589666</v>
-          </cell>
-          <cell r="J63">
-            <v>7598.78419452888</v>
-          </cell>
-          <cell r="K63">
-            <v>9498.4802431611</v>
-          </cell>
-          <cell r="L63">
-            <v>9498.4802431611</v>
-          </cell>
-          <cell r="M63">
-            <v>5699.08814589666</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="B65">
-            <v>0</v>
-          </cell>
-          <cell r="C65">
-            <v>0</v>
-          </cell>
-          <cell r="D65">
-            <v>0</v>
-          </cell>
-          <cell r="E65">
-            <v>0</v>
-          </cell>
-          <cell r="F65">
-            <v>0</v>
-          </cell>
-          <cell r="G65">
-            <v>0</v>
-          </cell>
-          <cell r="H65">
-            <v>0</v>
-          </cell>
-          <cell r="I65">
-            <v>1196.8085106383</v>
-          </cell>
-          <cell r="J65">
-            <v>1595.74468085106</v>
-          </cell>
-          <cell r="K65">
-            <v>1994.68085106383</v>
-          </cell>
-          <cell r="L65">
-            <v>1994.68085106383</v>
-          </cell>
-          <cell r="M65">
-            <v>1196.8085106383</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="B72">
-            <v>0</v>
-          </cell>
-          <cell r="C72">
-            <v>0</v>
-          </cell>
-          <cell r="D72">
-            <v>0</v>
-          </cell>
-          <cell r="E72">
-            <v>0</v>
-          </cell>
-          <cell r="F72">
-            <v>0</v>
-          </cell>
-          <cell r="G72">
-            <v>0</v>
-          </cell>
-          <cell r="H72">
-            <v>21428571.4285714</v>
-          </cell>
-          <cell r="I72">
-            <v>64285714.2857143</v>
-          </cell>
-          <cell r="J72">
-            <v>89285714.2857143</v>
-          </cell>
-          <cell r="K72">
-            <v>89285714.2857143</v>
-          </cell>
-          <cell r="L72">
-            <v>71428571.4285714</v>
-          </cell>
-          <cell r="M72">
-            <v>21428571.4285714</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="B74">
-            <v>0</v>
-          </cell>
-          <cell r="C74">
-            <v>0</v>
-          </cell>
-          <cell r="D74">
-            <v>0</v>
-          </cell>
-          <cell r="E74">
-            <v>0</v>
-          </cell>
-          <cell r="F74">
-            <v>0</v>
-          </cell>
-          <cell r="G74">
-            <v>0</v>
-          </cell>
-          <cell r="H74">
-            <v>360000</v>
-          </cell>
-          <cell r="I74">
-            <v>1080000</v>
-          </cell>
-          <cell r="J74">
-            <v>1500000</v>
-          </cell>
-          <cell r="K74">
-            <v>1500000</v>
-          </cell>
-          <cell r="L74">
-            <v>1200000</v>
-          </cell>
-          <cell r="M74">
-            <v>360000</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="B76">
-            <v>0</v>
-          </cell>
-          <cell r="C76">
-            <v>0</v>
-          </cell>
-          <cell r="D76">
-            <v>0</v>
-          </cell>
-          <cell r="E76">
-            <v>0</v>
-          </cell>
-          <cell r="F76">
-            <v>0</v>
-          </cell>
-          <cell r="G76">
-            <v>0</v>
-          </cell>
-          <cell r="H76">
-            <v>55080</v>
-          </cell>
-          <cell r="I76">
-            <v>165240</v>
-          </cell>
-          <cell r="J76">
-            <v>229500</v>
-          </cell>
-          <cell r="K76">
-            <v>229500</v>
-          </cell>
-          <cell r="L76">
-            <v>183600</v>
-          </cell>
-          <cell r="M76">
-            <v>55080</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="B80">
-            <v>0</v>
-          </cell>
-          <cell r="C80">
-            <v>0</v>
-          </cell>
-          <cell r="D80">
-            <v>0</v>
-          </cell>
-          <cell r="E80">
-            <v>0</v>
-          </cell>
-          <cell r="F80">
-            <v>0</v>
-          </cell>
-          <cell r="G80">
-            <v>0</v>
-          </cell>
-          <cell r="H80">
-            <v>4559.27051671733</v>
-          </cell>
-          <cell r="I80">
-            <v>13677.811550152</v>
-          </cell>
-          <cell r="J80">
-            <v>18996.9604863222</v>
-          </cell>
-          <cell r="K80">
-            <v>18996.9604863222</v>
-          </cell>
-          <cell r="L80">
-            <v>15197.5683890578</v>
-          </cell>
-          <cell r="M80">
-            <v>4559.27051671733</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="B82">
-            <v>0</v>
-          </cell>
-          <cell r="C82">
-            <v>0</v>
-          </cell>
-          <cell r="D82">
-            <v>0</v>
-          </cell>
-          <cell r="E82">
-            <v>0</v>
-          </cell>
-          <cell r="F82">
-            <v>0</v>
-          </cell>
-          <cell r="G82">
-            <v>0</v>
-          </cell>
-          <cell r="H82">
-            <v>957.446808510638</v>
-          </cell>
-          <cell r="I82">
-            <v>2872.34042553191</v>
-          </cell>
-          <cell r="J82">
-            <v>3989.36170212766</v>
-          </cell>
-          <cell r="K82">
-            <v>3989.36170212766</v>
-          </cell>
-          <cell r="L82">
-            <v>3191.48936170213</v>
-          </cell>
-          <cell r="M82">
-            <v>957.446808510638</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="B89">
-            <v>0</v>
-          </cell>
-          <cell r="C89">
-            <v>0</v>
-          </cell>
-          <cell r="D89">
-            <v>0</v>
-          </cell>
-          <cell r="E89">
-            <v>0</v>
-          </cell>
-          <cell r="F89">
-            <v>0</v>
-          </cell>
-          <cell r="G89">
-            <v>0</v>
-          </cell>
-          <cell r="H89">
-            <v>21428571.4285714</v>
-          </cell>
-          <cell r="I89">
-            <v>35714285.7142857</v>
-          </cell>
-          <cell r="J89">
-            <v>32142857.1428571</v>
-          </cell>
-          <cell r="K89">
-            <v>32142857.1428571</v>
-          </cell>
-          <cell r="L89">
-            <v>32142857.1428571</v>
-          </cell>
-          <cell r="M89">
-            <v>25000000</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="B91">
-            <v>0</v>
-          </cell>
-          <cell r="C91">
-            <v>0</v>
-          </cell>
-          <cell r="D91">
-            <v>0</v>
-          </cell>
-          <cell r="E91">
-            <v>0</v>
-          </cell>
-          <cell r="F91">
-            <v>0</v>
-          </cell>
-          <cell r="G91">
-            <v>0</v>
-          </cell>
-          <cell r="H91">
-            <v>360000</v>
-          </cell>
-          <cell r="I91">
-            <v>600000</v>
-          </cell>
-          <cell r="J91">
-            <v>540000</v>
-          </cell>
-          <cell r="K91">
-            <v>540000</v>
-          </cell>
-          <cell r="L91">
-            <v>540000</v>
-          </cell>
-          <cell r="M91">
-            <v>420000</v>
-          </cell>
-        </row>
-        <row r="93">
-          <cell r="B93">
-            <v>0</v>
-          </cell>
-          <cell r="C93">
-            <v>0</v>
-          </cell>
-          <cell r="D93">
-            <v>0</v>
-          </cell>
-          <cell r="E93">
-            <v>0</v>
-          </cell>
-          <cell r="F93">
-            <v>0</v>
-          </cell>
-          <cell r="G93">
-            <v>0</v>
-          </cell>
-          <cell r="H93">
-            <v>36000</v>
-          </cell>
-          <cell r="I93">
-            <v>60000</v>
-          </cell>
-          <cell r="J93">
-            <v>54000</v>
-          </cell>
-          <cell r="K93">
-            <v>54000</v>
-          </cell>
-          <cell r="L93">
-            <v>54000</v>
-          </cell>
-          <cell r="M93">
-            <v>42000</v>
-          </cell>
-        </row>
-        <row r="97">
-          <cell r="B97">
-            <v>0</v>
-          </cell>
-          <cell r="C97">
-            <v>0</v>
-          </cell>
-          <cell r="D97">
-            <v>0</v>
-          </cell>
-          <cell r="E97">
-            <v>0</v>
-          </cell>
-          <cell r="F97">
-            <v>0</v>
-          </cell>
-          <cell r="G97">
-            <v>0</v>
-          </cell>
-          <cell r="H97">
-            <v>4559.27051671733</v>
-          </cell>
-          <cell r="I97">
-            <v>7598.78419452888</v>
-          </cell>
-          <cell r="J97">
-            <v>6838.90577507599</v>
-          </cell>
-          <cell r="K97">
-            <v>6838.90577507599</v>
-          </cell>
-          <cell r="L97">
-            <v>6838.90577507599</v>
-          </cell>
-          <cell r="M97">
-            <v>5319.14893617021</v>
-          </cell>
-        </row>
-        <row r="99">
-          <cell r="B99">
-            <v>0</v>
-          </cell>
-          <cell r="C99">
-            <v>0</v>
-          </cell>
-          <cell r="D99">
-            <v>0</v>
-          </cell>
-          <cell r="E99">
-            <v>0</v>
-          </cell>
-          <cell r="F99">
-            <v>0</v>
-          </cell>
-          <cell r="G99">
-            <v>0</v>
-          </cell>
-          <cell r="H99">
-            <v>957.446808510638</v>
-          </cell>
-          <cell r="I99">
-            <v>1595.74468085106</v>
-          </cell>
-          <cell r="J99">
-            <v>1436.17021276596</v>
-          </cell>
-          <cell r="K99">
-            <v>1436.17021276596</v>
-          </cell>
-          <cell r="L99">
-            <v>1436.17021276596</v>
-          </cell>
-          <cell r="M99">
-            <v>1117.02127659574</v>
           </cell>
         </row>
       </sheetData>
@@ -3626,7 +3652,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="3">
         <f>(F7+G7+H7)</f>
-        <v>188699.09</v>
+        <v>225633.990762419</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -3657,7 +3683,7 @@
       <c r="E5" s="6"/>
       <c r="F5" s="7">
         <f>(F7+G7+H7)/(F6+G6+H6)</f>
-        <v>0.552986463661553</v>
+        <v>0.661224930303339</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -3683,51 +3709,51 @@
         <v>24</v>
       </c>
       <c r="C6" s="10">
-        <f>[1]目标拆解!B42</f>
+        <f>[2]目标拆解!B42</f>
         <v>25963.6363636363</v>
       </c>
       <c r="D6" s="10">
-        <f>[1]目标拆解!C42</f>
+        <f>[2]目标拆解!C42</f>
         <v>57490.9090909092</v>
       </c>
       <c r="E6" s="10">
-        <f>[1]目标拆解!D42</f>
+        <f>[2]目标拆解!D42</f>
         <v>111272.727272727</v>
       </c>
       <c r="F6" s="10">
-        <f>[1]目标拆解!E42</f>
+        <f>[2]目标拆解!E42</f>
         <v>114981.818181818</v>
       </c>
       <c r="G6" s="10">
-        <f>[1]目标拆解!F42</f>
+        <f>[2]目标拆解!F42</f>
         <v>111272.727272727</v>
       </c>
       <c r="H6" s="10">
-        <f>[1]目标拆解!G42</f>
+        <f>[2]目标拆解!G42</f>
         <v>114981.818181818</v>
       </c>
       <c r="I6" s="10">
-        <f>[1]目标拆解!H42</f>
+        <f>[2]目标拆解!H42</f>
         <v>201218.181818182</v>
       </c>
       <c r="J6" s="10">
-        <f>[1]目标拆解!I42</f>
+        <f>[2]目标拆解!I42</f>
         <v>194727.272727272</v>
       </c>
       <c r="K6" s="10">
-        <f>[1]目标拆解!J42</f>
+        <f>[2]目标拆解!J42</f>
         <v>172472.727272727</v>
       </c>
       <c r="L6" s="10">
-        <f>[1]目标拆解!K42</f>
+        <f>[2]目标拆解!K42</f>
         <v>166909.09090909</v>
       </c>
       <c r="M6" s="10">
-        <f>[1]目标拆解!L42</f>
+        <f>[2]目标拆解!L42</f>
         <v>172472.727272727</v>
       </c>
       <c r="N6" s="10">
-        <f>[1]目标拆解!M42</f>
+        <f>[2]目标拆解!M42</f>
         <v>86236.3636363634</v>
       </c>
       <c r="O6" s="31">
@@ -3741,56 +3767,56 @@
         <v>25</v>
       </c>
       <c r="C7" s="13">
-        <f>'[1]月度数据汇总--女装'!C8</f>
+        <f>'[2]月度数据汇总--女装'!C8</f>
         <v>63564.22</v>
       </c>
       <c r="D7" s="13">
-        <f>'[1]月度数据汇总--女装'!D8</f>
+        <f>'[2]月度数据汇总--女装'!D8</f>
         <v>186252.86</v>
       </c>
       <c r="E7" s="13">
-        <f>'[1]月度数据汇总--女装'!E8</f>
+        <f>'[2]月度数据汇总--女装'!E8</f>
         <v>23902.22</v>
       </c>
       <c r="F7" s="13">
-        <f>'[1]月度数据汇总--女装'!F8</f>
+        <f>'[2]月度数据汇总--女装'!F8</f>
         <v>154982.1</v>
       </c>
       <c r="G7" s="13">
-        <f>'[1]月度数据汇总--女装'!G8</f>
-        <v>33716.99</v>
+        <f>'[2]月度数据汇总--女装'!G8</f>
+        <v>58803.505650204</v>
       </c>
       <c r="H7" s="13">
-        <f>'[1]月度数据汇总--女装'!H8</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H8</f>
+        <v>11848.3851122148</v>
       </c>
       <c r="I7" s="13">
-        <f>'[1]月度数据汇总--女装'!I8</f>
+        <f>'[2]月度数据汇总--女装'!I8</f>
         <v>0</v>
       </c>
       <c r="J7" s="13">
-        <f>'[1]月度数据汇总--女装'!J8</f>
+        <f>'[2]月度数据汇总--女装'!J8</f>
         <v>0</v>
       </c>
       <c r="K7" s="13">
-        <f>'[1]月度数据汇总--女装'!K8</f>
+        <f>'[2]月度数据汇总--女装'!K8</f>
         <v>0</v>
       </c>
       <c r="L7" s="13">
-        <f>'[1]月度数据汇总--女装'!L8</f>
+        <f>'[2]月度数据汇总--女装'!L8</f>
         <v>0</v>
       </c>
       <c r="M7" s="13">
-        <f>'[1]月度数据汇总--女装'!M8</f>
+        <f>'[2]月度数据汇总--女装'!M8</f>
         <v>0</v>
       </c>
       <c r="N7" s="13">
-        <f>'[1]月度数据汇总--女装'!N8</f>
+        <f>'[2]月度数据汇总--女装'!N8</f>
         <v>0</v>
       </c>
       <c r="O7" s="13">
         <f>SUM(C7:N7)</f>
-        <v>462418.39</v>
+        <v>499353.290762419</v>
       </c>
     </row>
     <row r="8" ht="15.6" spans="1:15">
@@ -3816,11 +3842,11 @@
       </c>
       <c r="G8" s="15">
         <f t="shared" si="0"/>
-        <v>0.30301216503268</v>
+        <v>0.528462877575364</v>
       </c>
       <c r="H8" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.103045727573026</v>
       </c>
       <c r="I8" s="15">
         <f t="shared" si="0"/>
@@ -3848,7 +3874,7 @@
       </c>
       <c r="O8" s="15">
         <f t="shared" si="0"/>
-        <v>0.302234241830066</v>
+        <v>0.326374699844719</v>
       </c>
     </row>
     <row r="9" ht="15.6" spans="1:15">
@@ -3874,51 +3900,51 @@
         <v>27</v>
       </c>
       <c r="C10" s="19">
-        <f>[1]目标拆解!B46</f>
+        <f>[2]目标拆解!B46</f>
         <v>2051.46239962488</v>
       </c>
       <c r="D10" s="19">
-        <f>[1]目标拆解!C46</f>
+        <f>[2]目标拆解!C46</f>
         <v>4542.52388488367</v>
       </c>
       <c r="E10" s="19">
-        <f>[1]目标拆解!D46</f>
+        <f>[2]目标拆解!D46</f>
         <v>8791.98171267802</v>
       </c>
       <c r="F10" s="19">
-        <f>[1]目标拆解!E46</f>
+        <f>[2]目标拆解!E46</f>
         <v>9085.0477697673</v>
       </c>
       <c r="G10" s="19">
-        <f>[1]目标拆解!F46</f>
+        <f>[2]目标拆解!F46</f>
         <v>8791.98171267802</v>
       </c>
       <c r="H10" s="19">
-        <f>[1]目标拆解!G46</f>
+        <f>[2]目标拆解!G46</f>
         <v>9085.0477697673</v>
       </c>
       <c r="I10" s="19">
-        <f>[1]目标拆解!H46</f>
+        <f>[2]目标拆解!H46</f>
         <v>15898.8335970928</v>
       </c>
       <c r="J10" s="19">
-        <f>[1]目标拆解!I46</f>
+        <f>[2]目标拆解!I46</f>
         <v>15385.9679971865</v>
       </c>
       <c r="K10" s="19">
-        <f>[1]目标拆解!J46</f>
+        <f>[2]目标拆解!J46</f>
         <v>13627.571654651</v>
       </c>
       <c r="L10" s="19">
-        <f>[1]目标拆解!K46</f>
+        <f>[2]目标拆解!K46</f>
         <v>13187.972569017</v>
       </c>
       <c r="M10" s="19">
-        <f>[1]目标拆解!L46</f>
+        <f>[2]目标拆解!L46</f>
         <v>13627.571654651</v>
       </c>
       <c r="N10" s="19">
-        <f>[1]目标拆解!M46</f>
+        <f>[2]目标拆解!M46</f>
         <v>6813.78582732546</v>
       </c>
       <c r="O10" s="38">
@@ -3932,56 +3958,56 @@
         <v>28</v>
       </c>
       <c r="C11" s="12">
-        <f>'[1]月度数据汇总--女装'!C9</f>
+        <f>'[2]月度数据汇总--女装'!C9</f>
         <v>3019</v>
       </c>
       <c r="D11" s="12">
-        <f>'[1]月度数据汇总--女装'!D9</f>
+        <f>'[2]月度数据汇总--女装'!D9</f>
         <v>10048</v>
       </c>
       <c r="E11" s="12">
-        <f>'[1]月度数据汇总--女装'!E9</f>
+        <f>'[2]月度数据汇总--女装'!E9</f>
         <v>5984</v>
       </c>
       <c r="F11" s="12">
-        <f>'[1]月度数据汇总--女装'!F9</f>
+        <f>'[2]月度数据汇总--女装'!F9</f>
         <v>11196</v>
       </c>
       <c r="G11" s="12">
-        <f>'[1]月度数据汇总--女装'!G9</f>
-        <v>4045</v>
+        <f>'[2]月度数据汇总--女装'!G9</f>
+        <v>7971</v>
       </c>
       <c r="H11" s="12">
-        <f>'[1]月度数据汇总--女装'!H9</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H9</f>
+        <v>1339</v>
       </c>
       <c r="I11" s="12">
-        <f>'[1]月度数据汇总--女装'!I9</f>
+        <f>'[2]月度数据汇总--女装'!I9</f>
         <v>0</v>
       </c>
       <c r="J11" s="12">
-        <f>'[1]月度数据汇总--女装'!J9</f>
+        <f>'[2]月度数据汇总--女装'!J9</f>
         <v>0</v>
       </c>
       <c r="K11" s="12">
-        <f>'[1]月度数据汇总--女装'!K9</f>
+        <f>'[2]月度数据汇总--女装'!K9</f>
         <v>0</v>
       </c>
       <c r="L11" s="12">
-        <f>'[1]月度数据汇总--女装'!L9</f>
+        <f>'[2]月度数据汇总--女装'!L9</f>
         <v>0</v>
       </c>
       <c r="M11" s="12">
-        <f>'[1]月度数据汇总--女装'!M9</f>
+        <f>'[2]月度数据汇总--女装'!M9</f>
         <v>0</v>
       </c>
       <c r="N11" s="12">
-        <f>'[1]月度数据汇总--女装'!N9</f>
+        <f>'[2]月度数据汇总--女装'!N9</f>
         <v>0</v>
       </c>
       <c r="O11" s="12">
         <f t="shared" si="1"/>
-        <v>34292</v>
+        <v>39557</v>
       </c>
     </row>
     <row r="12" ht="15.6" spans="1:15">
@@ -4007,11 +4033,11 @@
       </c>
       <c r="G12" s="15">
         <f t="shared" si="2"/>
-        <v>0.460078300000001</v>
+        <v>0.906621540000002</v>
       </c>
       <c r="H12" s="15">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.147385025806452</v>
       </c>
       <c r="I12" s="15">
         <f t="shared" si="2"/>
@@ -4039,7 +4065,7 @@
       </c>
       <c r="O12" s="15">
         <f t="shared" si="2"/>
-        <v>0.283663424</v>
+        <v>0.327215504</v>
       </c>
     </row>
     <row r="13" ht="15.6" spans="1:15">
@@ -4065,51 +4091,51 @@
         <v>30</v>
       </c>
       <c r="C14" s="20">
-        <f>[1]目标拆解!B31</f>
+        <f>[2]目标拆解!B31</f>
         <v>361.057382333979</v>
       </c>
       <c r="D14" s="20">
-        <f>[1]目标拆解!C31</f>
+        <f>[2]目标拆解!C31</f>
         <v>799.484203739525</v>
       </c>
       <c r="E14" s="20">
-        <f>[1]目标拆解!D31</f>
+        <f>[2]目标拆解!D31</f>
         <v>1547.38878143133</v>
       </c>
       <c r="F14" s="20">
-        <f>[1]目标拆解!E31</f>
+        <f>[2]目标拆解!E31</f>
         <v>1598.96840747904</v>
       </c>
       <c r="G14" s="20">
-        <f>[1]目标拆解!F31</f>
+        <f>[2]目标拆解!F31</f>
         <v>1547.38878143133</v>
       </c>
       <c r="H14" s="20">
-        <f>[1]目标拆解!G31</f>
+        <f>[2]目标拆解!G31</f>
         <v>1598.96840747904</v>
       </c>
       <c r="I14" s="20">
-        <f>[1]目标拆解!H31</f>
+        <f>[2]目标拆解!H31</f>
         <v>2798.19471308834</v>
       </c>
       <c r="J14" s="20">
-        <f>[1]目标拆解!I31</f>
+        <f>[2]目标拆解!I31</f>
         <v>2707.93036750483</v>
       </c>
       <c r="K14" s="20">
-        <f>[1]目标拆解!J31</f>
+        <f>[2]目标拆解!J31</f>
         <v>2398.45261121857</v>
       </c>
       <c r="L14" s="20">
-        <f>[1]目标拆解!K31</f>
+        <f>[2]目标拆解!K31</f>
         <v>2321.083172147</v>
       </c>
       <c r="M14" s="20">
-        <f>[1]目标拆解!L31</f>
+        <f>[2]目标拆解!L31</f>
         <v>2398.45261121857</v>
       </c>
       <c r="N14" s="20">
-        <f>[1]目标拆解!M31</f>
+        <f>[2]目标拆解!M31</f>
         <v>1199.22630560928</v>
       </c>
       <c r="O14" s="38">
@@ -4123,56 +4149,56 @@
         <v>31</v>
       </c>
       <c r="C15" s="12">
-        <f>'[1]月度数据汇总--女装'!C10</f>
+        <f>'[2]月度数据汇总--女装'!C10</f>
         <v>782</v>
       </c>
       <c r="D15" s="12">
-        <f>'[1]月度数据汇总--女装'!D10</f>
+        <f>'[2]月度数据汇总--女装'!D10</f>
         <v>2400</v>
       </c>
       <c r="E15" s="12">
-        <f>'[1]月度数据汇总--女装'!E10</f>
+        <f>'[2]月度数据汇总--女装'!E10</f>
         <v>1177</v>
       </c>
       <c r="F15" s="12">
-        <f>'[1]月度数据汇总--女装'!F10</f>
+        <f>'[2]月度数据汇总--女装'!F10</f>
         <v>2441</v>
       </c>
       <c r="G15" s="12">
-        <f>'[1]月度数据汇总--女装'!G10</f>
-        <v>887</v>
+        <f>'[2]月度数据汇总--女装'!G10</f>
+        <v>1758</v>
       </c>
       <c r="H15" s="12">
-        <f>'[1]月度数据汇总--女装'!H10</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H10</f>
+        <v>446</v>
       </c>
       <c r="I15" s="12">
-        <f>'[1]月度数据汇总--女装'!I10</f>
+        <f>'[2]月度数据汇总--女装'!I10</f>
         <v>0</v>
       </c>
       <c r="J15" s="12">
-        <f>'[1]月度数据汇总--女装'!J10</f>
+        <f>'[2]月度数据汇总--女装'!J10</f>
         <v>0</v>
       </c>
       <c r="K15" s="12">
-        <f>'[1]月度数据汇总--女装'!K10</f>
+        <f>'[2]月度数据汇总--女装'!K10</f>
         <v>0</v>
       </c>
       <c r="L15" s="12">
-        <f>'[1]月度数据汇总--女装'!L10</f>
+        <f>'[2]月度数据汇总--女装'!L10</f>
         <v>0</v>
       </c>
       <c r="M15" s="12">
-        <f>'[1]月度数据汇总--女装'!M10</f>
+        <f>'[2]月度数据汇总--女装'!M10</f>
         <v>0</v>
       </c>
       <c r="N15" s="12">
-        <f>'[1]月度数据汇总--女装'!N10</f>
+        <f>'[2]月度数据汇总--女装'!N10</f>
         <v>0</v>
       </c>
       <c r="O15" s="12">
         <f t="shared" si="1"/>
-        <v>7687</v>
+        <v>9004</v>
       </c>
     </row>
     <row r="16" ht="15.6" spans="1:15">
@@ -4198,11 +4224,11 @@
       </c>
       <c r="G16" s="15">
         <f t="shared" si="3"/>
-        <v>0.573223750000002</v>
+        <v>1.1361075</v>
       </c>
       <c r="H16" s="15">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.278929838709678</v>
       </c>
       <c r="I16" s="15">
         <f t="shared" si="3"/>
@@ -4230,7 +4256,7 @@
       </c>
       <c r="O16" s="15">
         <f t="shared" si="3"/>
-        <v>0.361289</v>
+        <v>0.423188</v>
       </c>
     </row>
     <row r="17" ht="15.6" spans="1:15">
@@ -4256,51 +4282,51 @@
         <v>33</v>
       </c>
       <c r="C18" s="22">
-        <f>[1]目标拆解!B38</f>
+        <f>[2]目标拆解!B38</f>
         <v>9641873.27823693</v>
       </c>
       <c r="D18" s="22">
-        <f>[1]目标拆解!C38</f>
+        <f>[2]目标拆解!C38</f>
         <v>21349862.2589532</v>
       </c>
       <c r="E18" s="22">
-        <f>[1]目标拆解!D38</f>
+        <f>[2]目标拆解!D38</f>
         <v>41322314.0495867</v>
       </c>
       <c r="F18" s="22">
-        <f>[1]目标拆解!E38</f>
+        <f>[2]目标拆解!E38</f>
         <v>42699724.5179063</v>
       </c>
       <c r="G18" s="22">
-        <f>[1]目标拆解!F38</f>
+        <f>[2]目标拆解!F38</f>
         <v>41322314.0495867</v>
       </c>
       <c r="H18" s="22">
-        <f>[1]目标拆解!G38</f>
+        <f>[2]目标拆解!G38</f>
         <v>42699724.5179063</v>
       </c>
       <c r="I18" s="22">
-        <f>[1]目标拆解!H38</f>
+        <f>[2]目标拆解!H38</f>
         <v>74724517.9063364</v>
       </c>
       <c r="J18" s="22">
-        <f>[1]目标拆解!I38</f>
+        <f>[2]目标拆解!I38</f>
         <v>72314049.5867767</v>
       </c>
       <c r="K18" s="22">
-        <f>[1]目标拆解!J38</f>
+        <f>[2]目标拆解!J38</f>
         <v>64049586.7768597</v>
       </c>
       <c r="L18" s="22">
-        <f>[1]目标拆解!K38</f>
+        <f>[2]目标拆解!K38</f>
         <v>61983471.0743801</v>
       </c>
       <c r="M18" s="22">
-        <f>[1]目标拆解!L38</f>
+        <f>[2]目标拆解!L38</f>
         <v>64049586.7768597</v>
       </c>
       <c r="N18" s="22">
-        <f>[1]目标拆解!M38</f>
+        <f>[2]目标拆解!M38</f>
         <v>32024793.3884297</v>
       </c>
       <c r="O18" s="34">
@@ -4314,56 +4340,56 @@
         <v>34</v>
       </c>
       <c r="C19" s="23">
-        <f>'[1]月度数据汇总--女装'!C11</f>
+        <f>'[2]月度数据汇总--女装'!C11</f>
         <v>17294018</v>
       </c>
       <c r="D19" s="23">
-        <f>'[1]月度数据汇总--女装'!D11</f>
+        <f>'[2]月度数据汇总--女装'!D11</f>
         <v>50353143</v>
       </c>
       <c r="E19" s="23">
-        <f>'[1]月度数据汇总--女装'!E11</f>
+        <f>'[2]月度数据汇总--女装'!E11</f>
         <v>30943005</v>
       </c>
       <c r="F19" s="23">
-        <f>'[1]月度数据汇总--女装'!F11</f>
+        <f>'[2]月度数据汇总--女装'!F11</f>
         <v>56092797</v>
       </c>
       <c r="G19" s="23">
-        <f>'[1]月度数据汇总--女装'!G11</f>
-        <v>18377548</v>
+        <f>'[2]月度数据汇总--女装'!G11</f>
+        <v>36922189</v>
       </c>
       <c r="H19" s="23">
-        <f>'[1]月度数据汇总--女装'!H11</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H11</f>
+        <v>8733473</v>
       </c>
       <c r="I19" s="23">
-        <f>'[1]月度数据汇总--女装'!I11</f>
+        <f>'[2]月度数据汇总--女装'!I11</f>
         <v>0</v>
       </c>
       <c r="J19" s="23">
-        <f>'[1]月度数据汇总--女装'!J11</f>
+        <f>'[2]月度数据汇总--女装'!J11</f>
         <v>0</v>
       </c>
       <c r="K19" s="23">
-        <f>'[1]月度数据汇总--女装'!K11</f>
+        <f>'[2]月度数据汇总--女装'!K11</f>
         <v>0</v>
       </c>
       <c r="L19" s="23">
-        <f>'[1]月度数据汇总--女装'!L11</f>
+        <f>'[2]月度数据汇总--女装'!L11</f>
         <v>0</v>
       </c>
       <c r="M19" s="23">
-        <f>'[1]月度数据汇总--女装'!M11</f>
+        <f>'[2]月度数据汇总--女装'!M11</f>
         <v>0</v>
       </c>
       <c r="N19" s="23">
-        <f>'[1]月度数据汇总--女装'!N11</f>
+        <f>'[2]月度数据汇总--女装'!N11</f>
         <v>0</v>
       </c>
       <c r="O19" s="23">
         <f>SUM(C19:N19)</f>
-        <v>173060511</v>
+        <v>200338625</v>
       </c>
     </row>
     <row r="20" ht="15.6" spans="1:15">
@@ -4389,11 +4415,11 @@
       </c>
       <c r="G20" s="15">
         <f t="shared" si="4"/>
-        <v>0.444736661600001</v>
+        <v>0.893516973800002</v>
       </c>
       <c r="H20" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.20453230316129</v>
       </c>
       <c r="I20" s="15">
         <f t="shared" si="4"/>
@@ -4421,7 +4447,7 @@
       </c>
       <c r="O20" s="15">
         <f t="shared" si="4"/>
-        <v>0.30458649936</v>
+        <v>0.35259598</v>
       </c>
     </row>
     <row r="21" ht="15.6" spans="1:15">
@@ -4447,51 +4473,51 @@
         <v>36</v>
       </c>
       <c r="C22" s="24">
-        <f>[1]目标拆解!B40</f>
+        <f>[2]目标拆解!B40</f>
         <v>169696.96969697</v>
       </c>
       <c r="D22" s="24">
-        <f>[1]目标拆解!C40</f>
+        <f>[2]目标拆解!C40</f>
         <v>375757.575757577</v>
       </c>
       <c r="E22" s="24">
-        <f>[1]目标拆解!D40</f>
+        <f>[2]目标拆解!D40</f>
         <v>727272.727272726</v>
       </c>
       <c r="F22" s="24">
-        <f>[1]目标拆解!E40</f>
+        <f>[2]目标拆解!E40</f>
         <v>751515.151515151</v>
       </c>
       <c r="G22" s="24">
-        <f>[1]目标拆解!F40</f>
+        <f>[2]目标拆解!F40</f>
         <v>727272.727272726</v>
       </c>
       <c r="H22" s="24">
-        <f>[1]目标拆解!G40</f>
+        <f>[2]目标拆解!G40</f>
         <v>751515.151515151</v>
       </c>
       <c r="I22" s="24">
-        <f>[1]目标拆解!H40</f>
+        <f>[2]目标拆解!H40</f>
         <v>1315151.51515151</v>
       </c>
       <c r="J22" s="24">
-        <f>[1]目标拆解!I40</f>
+        <f>[2]目标拆解!I40</f>
         <v>1272727.27272727</v>
       </c>
       <c r="K22" s="24">
-        <f>[1]目标拆解!J40</f>
+        <f>[2]目标拆解!J40</f>
         <v>1127272.72727273</v>
       </c>
       <c r="L22" s="24">
-        <f>[1]目标拆解!K40</f>
+        <f>[2]目标拆解!K40</f>
         <v>1090909.09090909</v>
       </c>
       <c r="M22" s="24">
-        <f>[1]目标拆解!L40</f>
+        <f>[2]目标拆解!L40</f>
         <v>1127272.72727273</v>
       </c>
       <c r="N22" s="24">
-        <f>[1]目标拆解!M40</f>
+        <f>[2]目标拆解!M40</f>
         <v>563636.363636362</v>
       </c>
       <c r="O22" s="31">
@@ -4505,56 +4531,56 @@
         <v>37</v>
       </c>
       <c r="C23" s="25">
-        <f>'[1]月度数据汇总--女装'!C12</f>
+        <f>'[2]月度数据汇总--女装'!C12</f>
         <v>324669.67</v>
       </c>
       <c r="D23" s="25">
-        <f>'[1]月度数据汇总--女装'!D12</f>
+        <f>'[2]月度数据汇总--女装'!D12</f>
         <v>1018496.8</v>
       </c>
       <c r="E23" s="25">
-        <f>'[1]月度数据汇总--女装'!E12</f>
+        <f>'[2]月度数据汇总--女装'!E12</f>
         <v>504766.74</v>
       </c>
       <c r="F23" s="25">
-        <f>'[1]月度数据汇总--女装'!F12</f>
+        <f>'[2]月度数据汇总--女装'!F12</f>
         <v>1069518.42</v>
       </c>
       <c r="G23" s="25">
-        <f>'[1]月度数据汇总--女装'!G12</f>
-        <v>401111.57</v>
+        <f>'[2]月度数据汇总--女装'!G12</f>
+        <v>797308.5406</v>
       </c>
       <c r="H23" s="25">
-        <f>'[1]月度数据汇总--女装'!H12</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H12</f>
+        <v>192321.5225</v>
       </c>
       <c r="I23" s="25">
-        <f>'[1]月度数据汇总--女装'!I12</f>
+        <f>'[2]月度数据汇总--女装'!I12</f>
         <v>0</v>
       </c>
       <c r="J23" s="25">
-        <f>'[1]月度数据汇总--女装'!J12</f>
+        <f>'[2]月度数据汇总--女装'!J12</f>
         <v>0</v>
       </c>
       <c r="K23" s="25">
-        <f>'[1]月度数据汇总--女装'!K12</f>
+        <f>'[2]月度数据汇总--女装'!K12</f>
         <v>0</v>
       </c>
       <c r="L23" s="25">
-        <f>'[1]月度数据汇总--女装'!L12</f>
+        <f>'[2]月度数据汇总--女装'!L12</f>
         <v>0</v>
       </c>
       <c r="M23" s="25">
-        <f>'[1]月度数据汇总--女装'!M12</f>
+        <f>'[2]月度数据汇总--女装'!M12</f>
         <v>0</v>
       </c>
       <c r="N23" s="25">
-        <f>'[1]月度数据汇总--女装'!N12</f>
+        <f>'[2]月度数据汇总--女装'!N12</f>
         <v>0</v>
       </c>
       <c r="O23" s="13">
         <f>SUM(C23:N23)</f>
-        <v>3318563.2</v>
+        <v>3907081.6931</v>
       </c>
     </row>
     <row r="24" ht="15.6" spans="1:15">
@@ -4580,11 +4606,11 @@
       </c>
       <c r="G24" s="15">
         <f t="shared" si="5"/>
-        <v>0.551528408750001</v>
+        <v>1.096299243325</v>
       </c>
       <c r="H24" s="15">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.255911703326613</v>
       </c>
       <c r="I24" s="15">
         <f t="shared" si="5"/>
@@ -4612,7 +4638,7 @@
       </c>
       <c r="O24" s="15">
         <f t="shared" si="5"/>
-        <v>0.33185632</v>
+        <v>0.39070816931</v>
       </c>
     </row>
     <row r="25" ht="15.6" spans="1:15">
@@ -4655,11 +4681,11 @@
       </c>
       <c r="G26" s="15">
         <f t="shared" si="6"/>
-        <v>0.727172818430402</v>
-      </c>
-      <c r="H26" s="15" t="e">
+        <v>0.730071346595945</v>
+      </c>
+      <c r="H26" s="15">
         <f t="shared" si="6"/>
-        <v>#DIV/0!</v>
+        <v>0.7247350474147</v>
       </c>
       <c r="I26" s="15" t="e">
         <f t="shared" si="6"/>
@@ -4687,7 +4713,7 @@
       </c>
       <c r="O26" s="15">
         <f t="shared" si="6"/>
-        <v>0.760303261788011</v>
+        <v>0.756220143950025</v>
       </c>
     </row>
     <row r="27" ht="15.6" spans="1:15">
@@ -4713,11 +4739,11 @@
       </c>
       <c r="G27" s="15">
         <f t="shared" si="7"/>
-        <v>0.780716934487021</v>
-      </c>
-      <c r="H27" s="15" t="e">
+        <v>0.779450508091833</v>
+      </c>
+      <c r="H27" s="15">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>0.666915608663182</v>
       </c>
       <c r="I27" s="15" t="e">
         <f t="shared" si="7"/>
@@ -4745,7 +4771,7 @@
       </c>
       <c r="O27" s="15">
         <f t="shared" si="7"/>
-        <v>0.775836929896186</v>
+        <v>0.772379098516065</v>
       </c>
     </row>
     <row r="28" ht="15.6" spans="1:15">
@@ -4771,11 +4797,11 @@
       </c>
       <c r="G28" s="39">
         <f t="shared" si="8"/>
-        <v>0.0840588816722489</v>
-      </c>
-      <c r="H28" s="39" t="e">
+        <v>0.0737525094186907</v>
+      </c>
+      <c r="H28" s="39">
         <f t="shared" si="8"/>
-        <v>#DIV/0!</v>
+        <v>0.0616071719805296</v>
       </c>
       <c r="I28" s="39" t="e">
         <f t="shared" si="8"/>
@@ -4803,7 +4829,7 @@
       </c>
       <c r="O28" s="39">
         <f t="shared" si="8"/>
-        <v>0.139342951190443</v>
+        <v>0.127807230558882</v>
       </c>
     </row>
     <row r="29" ht="15.6" spans="1:15">
@@ -4851,7 +4877,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{e006b730-45e0-44a0-9f5a-41fd5be88c85}</x14:id>
+          <x14:id>{88eca861-dbf7-497b-935a-d9fdcb8bb1d7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4862,7 +4888,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{e006b730-45e0-44a0-9f5a-41fd5be88c85}">
+          <x14:cfRule type="dataBar" id="{88eca861-dbf7-497b-935a-d9fdcb8bb1d7}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -5000,7 +5026,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="3">
         <f>(F7+G7+H7)</f>
-        <v>13481.55</v>
+        <v>-42989.3272272495</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -5031,7 +5057,7 @@
       <c r="E5" s="6"/>
       <c r="F5" s="7">
         <f>(F7+G7+H7)/(F6+G6+H6)</f>
-        <v>0.107941369856367</v>
+        <v>-0.344198320676251</v>
       </c>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -5057,51 +5083,51 @@
         <v>24</v>
       </c>
       <c r="C6" s="10">
-        <f>[1]目标拆解!B25</f>
+        <f>[2]目标拆解!B25</f>
         <v>9503.0303030303</v>
       </c>
       <c r="D6" s="10">
-        <f>[1]目标拆解!C25</f>
+        <f>[2]目标拆解!C25</f>
         <v>21042.4242424243</v>
       </c>
       <c r="E6" s="10">
-        <f>[1]目标拆解!D25</f>
+        <f>[2]目标拆解!D25</f>
         <v>40727.2727272727</v>
       </c>
       <c r="F6" s="10">
-        <f>[1]目标拆解!E25</f>
+        <f>[2]目标拆解!E25</f>
         <v>42084.8484848484</v>
       </c>
       <c r="G6" s="10">
-        <f>[1]目标拆解!F25</f>
+        <f>[2]目标拆解!F25</f>
         <v>40727.2727272727</v>
       </c>
       <c r="H6" s="10">
-        <f>[1]目标拆解!G25</f>
+        <f>[2]目标拆解!G25</f>
         <v>42084.8484848484</v>
       </c>
       <c r="I6" s="10">
-        <f>[1]目标拆解!H25</f>
+        <f>[2]目标拆解!H25</f>
         <v>73648.4848484848</v>
       </c>
       <c r="J6" s="10">
-        <f>[1]目标拆解!I25</f>
+        <f>[2]目标拆解!I25</f>
         <v>71272.7272727271</v>
       </c>
       <c r="K6" s="10">
-        <f>[1]目标拆解!J25</f>
+        <f>[2]目标拆解!J25</f>
         <v>63127.2727272727</v>
       </c>
       <c r="L6" s="10">
-        <f>[1]目标拆解!K25</f>
+        <f>[2]目标拆解!K25</f>
         <v>61090.9090909089</v>
       </c>
       <c r="M6" s="10">
-        <f>[1]目标拆解!L25</f>
+        <f>[2]目标拆解!L25</f>
         <v>63127.2727272727</v>
       </c>
       <c r="N6" s="10">
-        <f>[1]目标拆解!M25</f>
+        <f>[2]目标拆解!M25</f>
         <v>31563.6363636363</v>
       </c>
       <c r="O6" s="31">
@@ -5115,56 +5141,56 @@
         <v>25</v>
       </c>
       <c r="C7" s="37">
-        <f>'[1]月度数据汇总--女装'!C3</f>
+        <f>'[2]月度数据汇总--女装'!C3</f>
         <v>-6740.65</v>
       </c>
       <c r="D7" s="37">
-        <f>'[1]月度数据汇总--女装'!D3</f>
+        <f>'[2]月度数据汇总--女装'!D3</f>
         <v>106911.11</v>
       </c>
       <c r="E7" s="37">
-        <f>'[1]月度数据汇总--女装'!E3</f>
+        <f>'[2]月度数据汇总--女装'!E3</f>
         <v>10303.42</v>
       </c>
       <c r="F7" s="37">
-        <f>'[1]月度数据汇总--女装'!F3</f>
+        <f>'[2]月度数据汇总--女装'!F3</f>
         <v>27181.29</v>
       </c>
       <c r="G7" s="37">
-        <f>'[1]月度数据汇总--女装'!G3</f>
-        <v>-13699.74</v>
+        <f>'[2]月度数据汇总--女装'!G3</f>
+        <v>-76428.1812484271</v>
       </c>
       <c r="H7" s="37">
-        <f>'[1]月度数据汇总--女装'!H3</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H3</f>
+        <v>6257.5640211776</v>
       </c>
       <c r="I7" s="37">
-        <f>'[1]月度数据汇总--女装'!I3</f>
+        <f>'[2]月度数据汇总--女装'!I3</f>
         <v>0</v>
       </c>
       <c r="J7" s="37">
-        <f>'[1]月度数据汇总--女装'!J3</f>
+        <f>'[2]月度数据汇总--女装'!J3</f>
         <v>0</v>
       </c>
       <c r="K7" s="37">
-        <f>'[1]月度数据汇总--女装'!K3</f>
+        <f>'[2]月度数据汇总--女装'!K3</f>
         <v>0</v>
       </c>
       <c r="L7" s="37">
-        <f>'[1]月度数据汇总--女装'!L3</f>
+        <f>'[2]月度数据汇总--女装'!L3</f>
         <v>0</v>
       </c>
       <c r="M7" s="37">
-        <f>'[1]月度数据汇总--女装'!M3</f>
+        <f>'[2]月度数据汇总--女装'!M3</f>
         <v>0</v>
       </c>
       <c r="N7" s="37">
-        <f>'[1]月度数据汇总--女装'!N3</f>
+        <f>'[2]月度数据汇总--女装'!N3</f>
         <v>0</v>
       </c>
       <c r="O7" s="37">
         <f t="shared" si="0"/>
-        <v>123955.43</v>
+        <v>67484.5527727505</v>
       </c>
     </row>
     <row r="8" ht="15.6" spans="1:15">
@@ -5190,11 +5216,11 @@
       </c>
       <c r="G8" s="15">
         <f t="shared" si="1"/>
-        <v>-0.336377544642857</v>
+        <v>-1.87658480743906</v>
       </c>
       <c r="H8" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.148689237254364</v>
       </c>
       <c r="I8" s="15">
         <f t="shared" si="1"/>
@@ -5222,7 +5248,7 @@
       </c>
       <c r="O8" s="15">
         <f t="shared" si="1"/>
-        <v>0.221348982142857</v>
+        <v>0.12050812995134</v>
       </c>
     </row>
     <row r="9" ht="15.6" spans="1:15">
@@ -5248,7 +5274,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="19">
-        <f>[1]目标拆解!B29</f>
+        <f>[2]目标拆解!B29</f>
         <v>1805.28691166989</v>
       </c>
       <c r="D10" s="19">
@@ -5306,7 +5332,7 @@
         <v>28</v>
       </c>
       <c r="C11" s="12">
-        <f>'[1]月度数据汇总--女装'!C4</f>
+        <f>'[2]月度数据汇总--女装'!C4</f>
         <v>2362</v>
       </c>
       <c r="D11" s="12">
@@ -5439,51 +5465,51 @@
         <v>30</v>
       </c>
       <c r="C14" s="20">
-        <f>[1]目标拆解!B31</f>
+        <f>[2]目标拆解!B31</f>
         <v>361.057382333979</v>
       </c>
       <c r="D14" s="20">
-        <f>[1]目标拆解!C31</f>
+        <f>[2]目标拆解!C31</f>
         <v>799.484203739525</v>
       </c>
       <c r="E14" s="20">
-        <f>[1]目标拆解!D31</f>
+        <f>[2]目标拆解!D31</f>
         <v>1547.38878143133</v>
       </c>
       <c r="F14" s="20">
-        <f>[1]目标拆解!E31</f>
+        <f>[2]目标拆解!E31</f>
         <v>1598.96840747904</v>
       </c>
       <c r="G14" s="20">
-        <f>[1]目标拆解!F31</f>
+        <f>[2]目标拆解!F31</f>
         <v>1547.38878143133</v>
       </c>
       <c r="H14" s="20">
-        <f>[1]目标拆解!G31</f>
+        <f>[2]目标拆解!G31</f>
         <v>1598.96840747904</v>
       </c>
       <c r="I14" s="20">
-        <f>[1]目标拆解!H31</f>
+        <f>[2]目标拆解!H31</f>
         <v>2798.19471308834</v>
       </c>
       <c r="J14" s="20">
-        <f>[1]目标拆解!I31</f>
+        <f>[2]目标拆解!I31</f>
         <v>2707.93036750483</v>
       </c>
       <c r="K14" s="20">
-        <f>[1]目标拆解!J31</f>
+        <f>[2]目标拆解!J31</f>
         <v>2398.45261121857</v>
       </c>
       <c r="L14" s="20">
-        <f>[1]目标拆解!K31</f>
+        <f>[2]目标拆解!K31</f>
         <v>2321.083172147</v>
       </c>
       <c r="M14" s="20">
-        <f>[1]目标拆解!L31</f>
+        <f>[2]目标拆解!L31</f>
         <v>2398.45261121857</v>
       </c>
       <c r="N14" s="20">
-        <f>[1]目标拆解!M31</f>
+        <f>[2]目标拆解!M31</f>
         <v>1199.22630560928</v>
       </c>
       <c r="O14" s="38">
@@ -5497,56 +5523,56 @@
         <v>31</v>
       </c>
       <c r="C15" s="12">
-        <f>'[1]月度数据汇总--女装'!C5</f>
+        <f>'[2]月度数据汇总--女装'!C5</f>
         <v>481</v>
       </c>
       <c r="D15" s="12">
-        <f>'[1]月度数据汇总--女装'!D5</f>
+        <f>'[2]月度数据汇总--女装'!D5</f>
         <v>2002</v>
       </c>
       <c r="E15" s="12">
-        <f>'[1]月度数据汇总--女装'!E5</f>
+        <f>'[2]月度数据汇总--女装'!E5</f>
         <v>1121</v>
       </c>
       <c r="F15" s="12">
-        <f>'[1]月度数据汇总--女装'!F5</f>
+        <f>'[2]月度数据汇总--女装'!F5</f>
         <v>1147</v>
       </c>
       <c r="G15" s="12">
-        <f>'[1]月度数据汇总--女装'!G5</f>
-        <v>510</v>
+        <f>'[2]月度数据汇总--女装'!G5</f>
+        <v>991</v>
       </c>
       <c r="H15" s="12">
-        <f>'[1]月度数据汇总--女装'!H5</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H5</f>
+        <v>216</v>
       </c>
       <c r="I15" s="12">
-        <f>'[1]月度数据汇总--女装'!I5</f>
+        <f>'[2]月度数据汇总--女装'!I5</f>
         <v>0</v>
       </c>
       <c r="J15" s="12">
-        <f>'[1]月度数据汇总--女装'!J5</f>
+        <f>'[2]月度数据汇总--女装'!J5</f>
         <v>0</v>
       </c>
       <c r="K15" s="12">
-        <f>'[1]月度数据汇总--女装'!K5</f>
+        <f>'[2]月度数据汇总--女装'!K5</f>
         <v>0</v>
       </c>
       <c r="L15" s="12">
-        <f>'[1]月度数据汇总--女装'!L5</f>
+        <f>'[2]月度数据汇总--女装'!L5</f>
         <v>0</v>
       </c>
       <c r="M15" s="12">
-        <f>'[1]月度数据汇总--女装'!M5</f>
+        <f>'[2]月度数据汇总--女装'!M5</f>
         <v>0</v>
       </c>
       <c r="N15" s="12">
-        <f>'[1]月度数据汇总--女装'!N5</f>
+        <f>'[2]月度数据汇总--女装'!N5</f>
         <v>0</v>
       </c>
       <c r="O15" s="12">
         <f t="shared" si="3"/>
-        <v>5261</v>
+        <v>5958</v>
       </c>
     </row>
     <row r="16" ht="15.6" spans="1:15">
@@ -5572,11 +5598,11 @@
       </c>
       <c r="G16" s="15">
         <f t="shared" si="4"/>
-        <v>0.329587500000001</v>
+        <v>0.640433750000002</v>
       </c>
       <c r="H16" s="15">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.135087096774194</v>
       </c>
       <c r="I16" s="15">
         <f t="shared" si="4"/>
@@ -5604,7 +5630,7 @@
       </c>
       <c r="O16" s="15">
         <f t="shared" si="4"/>
-        <v>0.247267</v>
+        <v>0.280026</v>
       </c>
     </row>
     <row r="17" ht="15.6" spans="1:15">
@@ -5630,51 +5656,51 @@
         <v>33</v>
       </c>
       <c r="C18" s="22">
-        <f>[1]目标拆解!B21</f>
+        <f>[2]目标拆解!B21</f>
         <v>8484848.4848485</v>
       </c>
       <c r="D18" s="22">
-        <f>[1]目标拆解!C21</f>
+        <f>[2]目标拆解!C21</f>
         <v>18787878.7878789</v>
       </c>
       <c r="E18" s="22">
-        <f>[1]目标拆解!D21</f>
+        <f>[2]目标拆解!D21</f>
         <v>36363636.3636363</v>
       </c>
       <c r="F18" s="22">
-        <f>[1]目标拆解!E21</f>
+        <f>[2]目标拆解!E21</f>
         <v>37575757.5757575</v>
       </c>
       <c r="G18" s="22">
-        <f>[1]目标拆解!F21</f>
+        <f>[2]目标拆解!F21</f>
         <v>36363636.3636363</v>
       </c>
       <c r="H18" s="22">
-        <f>[1]目标拆解!G21</f>
+        <f>[2]目标拆解!G21</f>
         <v>37575757.5757575</v>
       </c>
       <c r="I18" s="22">
-        <f>[1]目标拆解!H21</f>
+        <f>[2]目标拆解!H21</f>
         <v>65757575.757576</v>
       </c>
       <c r="J18" s="22">
-        <f>[1]目标拆解!I21</f>
+        <f>[2]目标拆解!I21</f>
         <v>63636363.6363635</v>
       </c>
       <c r="K18" s="22">
-        <f>[1]目标拆解!J21</f>
+        <f>[2]目标拆解!J21</f>
         <v>56363636.3636365</v>
       </c>
       <c r="L18" s="22">
-        <f>[1]目标拆解!K21</f>
+        <f>[2]目标拆解!K21</f>
         <v>54545454.5454545</v>
       </c>
       <c r="M18" s="22">
-        <f>[1]目标拆解!L21</f>
+        <f>[2]目标拆解!L21</f>
         <v>56363636.3636365</v>
       </c>
       <c r="N18" s="22">
-        <f>[1]目标拆解!M21</f>
+        <f>[2]目标拆解!M21</f>
         <v>28181818.1818181</v>
       </c>
       <c r="O18" s="34">
@@ -5688,56 +5714,56 @@
         <v>34</v>
       </c>
       <c r="C19" s="23">
-        <f>'[1]月度数据汇总--女装'!C6</f>
+        <f>'[2]月度数据汇总--女装'!C6</f>
         <v>13160868</v>
       </c>
       <c r="D19" s="23">
-        <f>'[1]月度数据汇总--女装'!D6</f>
+        <f>'[2]月度数据汇总--女装'!D6</f>
         <v>52320625</v>
       </c>
       <c r="E19" s="23">
-        <f>'[1]月度数据汇总--女装'!E6</f>
+        <f>'[2]月度数据汇总--女装'!E6</f>
         <v>29482199</v>
       </c>
       <c r="F19" s="23">
-        <f>'[1]月度数据汇总--女装'!F6</f>
+        <f>'[2]月度数据汇总--女装'!F6</f>
         <v>32616432</v>
       </c>
       <c r="G19" s="23">
-        <f>'[1]月度数据汇总--女装'!G6</f>
-        <v>11981910</v>
+        <f>'[2]月度数据汇总--女装'!G6</f>
+        <v>22407232</v>
       </c>
       <c r="H19" s="23">
-        <f>'[1]月度数据汇总--女装'!H6</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H6</f>
+        <v>4613093</v>
       </c>
       <c r="I19" s="23">
-        <f>'[1]月度数据汇总--女装'!I6</f>
+        <f>'[2]月度数据汇总--女装'!I6</f>
         <v>0</v>
       </c>
       <c r="J19" s="23">
-        <f>'[1]月度数据汇总--女装'!J6</f>
+        <f>'[2]月度数据汇总--女装'!J6</f>
         <v>0</v>
       </c>
       <c r="K19" s="23">
-        <f>'[1]月度数据汇总--女装'!K6</f>
+        <f>'[2]月度数据汇总--女装'!K6</f>
         <v>0</v>
       </c>
       <c r="L19" s="23">
-        <f>'[1]月度数据汇总--女装'!L6</f>
+        <f>'[2]月度数据汇总--女装'!L6</f>
         <v>0</v>
       </c>
       <c r="M19" s="23">
-        <f>'[1]月度数据汇总--女装'!M6</f>
+        <f>'[2]月度数据汇总--女装'!M6</f>
         <v>0</v>
       </c>
       <c r="N19" s="23">
-        <f>'[1]月度数据汇总--女装'!N6</f>
+        <f>'[2]月度数据汇总--女装'!N6</f>
         <v>0</v>
       </c>
       <c r="O19" s="23">
         <f t="shared" si="3"/>
-        <v>139562034</v>
+        <v>154600449</v>
       </c>
     </row>
     <row r="20" ht="15.6" spans="1:15">
@@ -5763,11 +5789,11 @@
       </c>
       <c r="G20" s="15">
         <f t="shared" si="5"/>
-        <v>0.329502525000001</v>
+        <v>0.616198880000001</v>
       </c>
       <c r="H20" s="15">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.122767797580645</v>
       </c>
       <c r="I20" s="15">
         <f t="shared" si="5"/>
@@ -5795,7 +5821,7 @@
       </c>
       <c r="O20" s="15">
         <f t="shared" si="5"/>
-        <v>0.279124068</v>
+        <v>0.309200898</v>
       </c>
     </row>
     <row r="21" ht="15.6" spans="1:15">
@@ -5821,51 +5847,51 @@
         <v>36</v>
       </c>
       <c r="C22" s="24">
-        <f>[1]目标拆解!B23</f>
+        <f>[2]目标拆解!B23</f>
         <v>135757.575757576</v>
       </c>
       <c r="D22" s="24">
-        <f>[1]目标拆解!C23</f>
+        <f>[2]目标拆解!C23</f>
         <v>300606.060606061</v>
       </c>
       <c r="E22" s="24">
-        <f>[1]目标拆解!D23</f>
+        <f>[2]目标拆解!D23</f>
         <v>581818.181818181</v>
       </c>
       <c r="F22" s="24">
-        <f>[1]目标拆解!E23</f>
+        <f>[2]目标拆解!E23</f>
         <v>601212.12121212</v>
       </c>
       <c r="G22" s="24">
-        <f>[1]目标拆解!F23</f>
+        <f>[2]目标拆解!F23</f>
         <v>581818.181818181</v>
       </c>
       <c r="H22" s="24">
-        <f>[1]目标拆解!G23</f>
+        <f>[2]目标拆解!G23</f>
         <v>601212.12121212</v>
       </c>
       <c r="I22" s="24">
-        <f>[1]目标拆解!H23</f>
+        <f>[2]目标拆解!H23</f>
         <v>1052121.21212121</v>
       </c>
       <c r="J22" s="24">
-        <f>[1]目标拆解!I23</f>
+        <f>[2]目标拆解!I23</f>
         <v>1018181.81818182</v>
       </c>
       <c r="K22" s="24">
-        <f>[1]目标拆解!J23</f>
+        <f>[2]目标拆解!J23</f>
         <v>901818.181818182</v>
       </c>
       <c r="L22" s="24">
-        <f>[1]目标拆解!K23</f>
+        <f>[2]目标拆解!K23</f>
         <v>872727.27272727</v>
       </c>
       <c r="M22" s="24">
-        <f>[1]目标拆解!L23</f>
+        <f>[2]目标拆解!L23</f>
         <v>901818.181818182</v>
       </c>
       <c r="N22" s="24">
-        <f>[1]目标拆解!M23</f>
+        <f>[2]目标拆解!M23</f>
         <v>450909.090909089</v>
       </c>
       <c r="O22" s="31">
@@ -5879,56 +5905,56 @@
         <v>37</v>
       </c>
       <c r="C23" s="25">
-        <f>'[1]月度数据汇总--女装'!C7</f>
+        <f>'[2]月度数据汇总--女装'!C7</f>
         <v>197473.98</v>
       </c>
       <c r="D23" s="25">
-        <f>'[1]月度数据汇总--女装'!D7</f>
+        <f>'[2]月度数据汇总--女装'!D7</f>
         <v>878014.15</v>
       </c>
       <c r="E23" s="25">
-        <f>'[1]月度数据汇总--女装'!E7</f>
+        <f>'[2]月度数据汇总--女装'!E7</f>
         <v>493495.3</v>
       </c>
       <c r="F23" s="25">
-        <f>'[1]月度数据汇总--女装'!F7</f>
+        <f>'[2]月度数据汇总--女装'!F7</f>
         <v>550489.45</v>
       </c>
       <c r="G23" s="25">
-        <f>'[1]月度数据汇总--女装'!G7</f>
-        <v>238074.01</v>
+        <f>'[2]月度数据汇总--女装'!G7</f>
+        <v>460996.035</v>
       </c>
       <c r="H23" s="25">
-        <f>'[1]月度数据汇总--女装'!H7</f>
-        <v>0</v>
+        <f>'[2]月度数据汇总--女装'!H7</f>
+        <v>94048.8148</v>
       </c>
       <c r="I23" s="25">
-        <f>'[1]月度数据汇总--女装'!I7</f>
+        <f>'[2]月度数据汇总--女装'!I7</f>
         <v>0</v>
       </c>
       <c r="J23" s="25">
-        <f>'[1]月度数据汇总--女装'!J7</f>
+        <f>'[2]月度数据汇总--女装'!J7</f>
         <v>0</v>
       </c>
       <c r="K23" s="25">
-        <f>'[1]月度数据汇总--女装'!K7</f>
+        <f>'[2]月度数据汇总--女装'!K7</f>
         <v>0</v>
       </c>
       <c r="L23" s="25">
-        <f>'[1]月度数据汇总--女装'!L7</f>
+        <f>'[2]月度数据汇总--女装'!L7</f>
         <v>0</v>
       </c>
       <c r="M23" s="25">
-        <f>'[1]月度数据汇总--女装'!M7</f>
+        <f>'[2]月度数据汇总--女装'!M7</f>
         <v>0</v>
       </c>
       <c r="N23" s="25">
-        <f>'[1]月度数据汇总--女装'!N7</f>
+        <f>'[2]月度数据汇总--女装'!N7</f>
         <v>0</v>
       </c>
       <c r="O23" s="13">
         <f>SUM(C23:N23)</f>
-        <v>2357546.89</v>
+        <v>2674517.7298</v>
       </c>
     </row>
     <row r="24" ht="15.6" spans="1:15">
@@ -5954,11 +5980,11 @@
       </c>
       <c r="G24" s="15">
         <f t="shared" si="6"/>
-        <v>0.409189704687501</v>
+        <v>0.792336935156251</v>
       </c>
       <c r="H24" s="15">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>0.156432000423387</v>
       </c>
       <c r="I24" s="15">
         <f t="shared" si="6"/>
@@ -5986,7 +6012,7 @@
       </c>
       <c r="O24" s="15">
         <f t="shared" si="6"/>
-        <v>0.29469336125</v>
+        <v>0.334314716225</v>
       </c>
     </row>
     <row r="25" ht="15.6" spans="1:15">
@@ -6029,11 +6055,11 @@
       </c>
       <c r="G26" s="15">
         <f t="shared" si="7"/>
-        <v>0.751631824558856</v>
-      </c>
-      <c r="H26" s="15" t="e">
+        <v>0.742830777246382</v>
+      </c>
+      <c r="H26" s="15">
         <f t="shared" si="7"/>
-        <v>#DIV/0!</v>
+        <v>0.745157926579846</v>
       </c>
       <c r="I26" s="15" t="e">
         <f t="shared" si="7"/>
@@ -6061,7 +6087,7 @@
       </c>
       <c r="O26" s="15">
         <f t="shared" si="7"/>
-        <v>0.788844177170705</v>
+        <v>0.783755662815054</v>
       </c>
     </row>
     <row r="27" ht="15.6" spans="1:15">
@@ -6087,7 +6113,7 @@
       </c>
       <c r="G27" s="15">
         <f t="shared" si="8"/>
-        <v>0.794603302456706</v>
+        <v>0.600886024969795</v>
       </c>
       <c r="H27" s="15" t="e">
         <f t="shared" si="8"/>
@@ -6119,7 +6145,7 @@
       </c>
       <c r="O27" s="15">
         <f t="shared" si="8"/>
-        <v>0.804967562557924</v>
+        <v>0.779128822984245</v>
       </c>
     </row>
     <row r="28" ht="15.6" spans="1:15">
@@ -6145,11 +6171,11 @@
       </c>
       <c r="G28" s="15">
         <f t="shared" si="9"/>
-        <v>-0.0575440385113856</v>
-      </c>
-      <c r="H28" s="15" t="e">
+        <v>-0.16578923775001</v>
+      </c>
+      <c r="H28" s="15">
         <f t="shared" si="9"/>
-        <v>#DIV/0!</v>
+        <v>0.0665352778180635</v>
       </c>
       <c r="I28" s="15" t="e">
         <f t="shared" si="9"/>
@@ -6177,7 +6203,7 @@
       </c>
       <c r="O28" s="15">
         <f t="shared" si="9"/>
-        <v>0.052578139813796</v>
+        <v>0.0252324192959442</v>
       </c>
     </row>
     <row r="29" ht="15.6" spans="1:15">
@@ -6225,7 +6251,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{714db6b9-3c84-4ebc-a780-d4747a9f38b8}</x14:id>
+          <x14:id>{b9ae6f34-c397-4483-86d9-45e556bad888}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -6236,7 +6262,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{714db6b9-3c84-4ebc-a780-d4747a9f38b8}">
+          <x14:cfRule type="dataBar" id="{b9ae6f34-c397-4483-86d9-45e556bad888}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -7598,7 +7624,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0f63a89d-f99c-4965-8e07-e7d5102966ba}</x14:id>
+          <x14:id>{eb8194ac-8435-4a6f-b1cb-8c8ac086be17}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -7609,7 +7635,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0f63a89d-f99c-4965-8e07-e7d5102966ba}">
+          <x14:cfRule type="dataBar" id="{eb8194ac-8435-4a6f-b1cb-8c8ac086be17}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -8969,7 +8995,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0904f572-004a-4a4d-bd74-55e55912aad2}</x14:id>
+          <x14:id>{5db08292-1cb6-4237-b546-af9cb44ef86b}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8980,7 +9006,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0904f572-004a-4a4d-bd74-55e55912aad2}">
+          <x14:cfRule type="dataBar" id="{5db08292-1cb6-4237-b546-af9cb44ef86b}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10340,7 +10366,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8f2ad983-3ea2-47d4-a8b8-6ffb91a3edf2}</x14:id>
+          <x14:id>{c5d2fffd-f391-4d7c-b26a-c029cc24ee7a}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10351,7 +10377,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8f2ad983-3ea2-47d4-a8b8-6ffb91a3edf2}">
+          <x14:cfRule type="dataBar" id="{c5d2fffd-f391-4d7c-b26a-c029cc24ee7a}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>
@@ -10367,4 +10393,18 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<NetdiskSupbooks xmlns="http://www.wps.cn/et/2019/netdiskSupbooks">
+  <NetdiskSupbook Target="file:///C:\Users\12139\WPSDrive\1725300681\WPS企业云盘\瑞安市水滴电子商务有限公司\团队文档\俄罗斯运营二部\俄罗斯运营二部--女装项目\2026女装年规_终版%20-%20所有女装店.xlsx" FileId="535888469621" NetdiskName="yunwps"/>
+</NetdiskSupbooks>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CA11897-456E-43AF-AC28-93E1BBEC0A59}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.wps.cn/et/2019/netdiskSupbooks"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>